<commit_message>
Ajustar TO-BE segun feedback: matriz con nombres y propuestas como solucion
- Matriz de Similitud: cada celda muestra "codigo — nombre de tarea"
  (antes solo el codigo) para validar las agrupaciones a la vista
- Propuestas: descripciones reescritas (62/62) para plantear la solucion,
  no repetir la necesidad del grupo
- Hoja Propuestas simplificada: se retiran columnas Anclas, Hallazgos RX
  y Aliado experto; la trazabilidad queda en propuestas.json
- xlsx regenerado

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Output/I.M.O/TO-BE/Matriz_y_Propuestas.xlsx
+++ b/Output/I.M.O/TO-BE/Matriz_y_Propuestas.xlsx
@@ -66,19 +66,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="38" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="16" customWidth="1"/>
-    <col min="13" max="13" width="16" customWidth="1"/>
-    <col min="14" max="14" width="16" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="30" customWidth="1"/>
+    <col min="11" max="11" width="30" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="30" customWidth="1"/>
+    <col min="14" max="14" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -171,7 +171,7 @@
       </c>
       <c r="D2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COM-1.1</t>
+          <t xml:space="preserve">COM-1.1 — Creacion de proveedores nuevos</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="2">
@@ -201,7 +201,7 @@
       </c>
       <c r="J2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.5.1</t>
+          <t xml:space="preserve">CCS-4.5.1 — Creacion de proveedores en Odoo</t>
         </is>
       </c>
       <c r="K2" t="inlineStr" s="2">
@@ -243,7 +243,7 @@
       </c>
       <c r="D3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COM-1.2</t>
+          <t xml:space="preserve">COM-1.2 — Creacion de productos</t>
         </is>
       </c>
       <c r="E3" t="inlineStr" s="2">
@@ -273,7 +273,9 @@
       </c>
       <c r="J3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.5.2, CCS-4.4.5, CCS-4.4.6</t>
+          <t xml:space="preserve">CCS-4.5.2 — Creacion de productos en Odoo
+CCS-4.4.5 — Revision de categorias contables en Odoo
+CCS-4.4.6 — Revision de cuentas contables en facturas de compra</t>
         </is>
       </c>
       <c r="K3" t="inlineStr" s="2">
@@ -283,12 +285,14 @@
       </c>
       <c r="L3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-13.1, AFL-13.2, AFL-13.5</t>
+          <t xml:space="preserve">AFL-13.1 — Creacion de productos en Odoo
+AFL-13.2 — Creacion de productos en Cloudbeds
+AFL-13.5 — Creacion de productos en Poster</t>
         </is>
       </c>
       <c r="M3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-1.4.5</t>
+          <t xml:space="preserve">GHO-1.4.5 — Actualizacion de lista de precios al publico</t>
         </is>
       </c>
       <c r="N3" t="inlineStr" s="2">
@@ -315,7 +319,8 @@
       </c>
       <c r="D4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COM-1.3, COM-4</t>
+          <t xml:space="preserve">COM-1.3 — Comparacion de precios y seleccion de proveedor
+COM-4 — Gestion de acuerdos marco con proveedores recurrentes</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="2">
@@ -335,12 +340,12 @@
       </c>
       <c r="H4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">BAR-4.5</t>
+          <t xml:space="preserve">BAR-4.5 — Solicitud de compra cuando almacen no tiene el producto</t>
         </is>
       </c>
       <c r="I4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COC-4.5</t>
+          <t xml:space="preserve">COC-4.5 — Solicitud de compra cuando almacen no tiene el producto</t>
         </is>
       </c>
       <c r="J4" t="inlineStr" s="2">
@@ -350,7 +355,7 @@
       </c>
       <c r="K4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-1.2</t>
+          <t xml:space="preserve">AFJ-1.2 — Solicitud de pedidos de compras excepcionales</t>
         </is>
       </c>
       <c r="L4" t="inlineStr" s="2">
@@ -365,7 +370,7 @@
       </c>
       <c r="N4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OPE-3.6</t>
+          <t xml:space="preserve">OPE-3.6 — Solicitud de compra de suministros y materiales</t>
         </is>
       </c>
     </row>
@@ -387,7 +392,12 @@
       </c>
       <c r="D5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COM-Alm-1.1, COM-Alm-1.2, COM-Alm-1.3, COM-Alm-1.4, COM-Alm-1.5, COM-Alm-1.13</t>
+          <t xml:space="preserve">COM-Alm-1.1 — Conteo fisico de mercancias para determinar pedidos semanales
+COM-Alm-1.2 — Planificacion y requisicion de reposicion de productos
+COM-Alm-1.3 — Atencion a solicitudes de suministros de departamentos internos
+COM-Alm-1.4 — Aprobacion de pedidos por Gerencia General
+COM-Alm-1.5 — Envio de pedidos aprobados al departamento de Compras
+COM-Alm-1.13 — Planificacion y coordinacion de pedidos para fines de semana</t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="2">
@@ -402,17 +412,21 @@
       </c>
       <c r="G5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CAJ-3.2, CAJ-3.3, CAJ-3.4</t>
+          <t xml:space="preserve">CAJ-3.2 — Solicitud de requisicion de productos a almacen general
+CAJ-3.3 — Llenado de formato de requisicion
+CAJ-3.4 — Solicitud de firma a Gerencia</t>
         </is>
       </c>
       <c r="H5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">BAR-4.2, BAR-4.3</t>
+          <t xml:space="preserve">BAR-4.2 — Relleno de formato de requisiciones
+BAR-4.3 — Solicitud de firma de requisicion a Gerencia de Operaciones</t>
         </is>
       </c>
       <c r="I5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COC-4.2, COC-4.3</t>
+          <t xml:space="preserve">COC-4.2 — Relleno de formato de requisiciones
+COC-4.3 — Solicitud de firma de requisicion a Gerencia / Jefe de cocina</t>
         </is>
       </c>
       <c r="J5" t="inlineStr" s="2">
@@ -422,22 +436,25 @@
       </c>
       <c r="K5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-8.1</t>
+          <t xml:space="preserve">AFJ-8.1 — Realizar oficios, requisiciones, inventarios y listas de personal</t>
         </is>
       </c>
       <c r="L5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-14.1</t>
+          <t xml:space="preserve">AFL-14.1 — Solicitud de articulos de oficina y mercancia a compras</t>
         </is>
       </c>
       <c r="M5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-3.5, GHO-4.1, GHO-5.1</t>
+          <t xml:space="preserve">GHO-3.5 — Firma y validacion semanal de requisiciones para Almacen (A&amp;B)
+GHO-4.1 — Firma y control de requisiciones semanales (Ama de Llaves)
+GHO-5.1 — Firma y control de requisiciones semanales (Lavanderia)</t>
         </is>
       </c>
       <c r="N5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OPE-3.3, OPE-4.4</t>
+          <t xml:space="preserve">OPE-3.3 — Solicitud de insumos a almacen
+OPE-4.4 — Solicitud de herramientas y materiales a Richard en el taller</t>
         </is>
       </c>
     </row>
@@ -459,7 +476,10 @@
       </c>
       <c r="D6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COM-Alm-1.6, COM-Alm-1.7, COM-Alm-1.8, COM-Alm-1.9</t>
+          <t xml:space="preserve">COM-Alm-1.6 — Verificacion de pedidos en transito
+COM-Alm-1.7 — Recepcion fisica y en sistema de mercancia de proveedores
+COM-Alm-1.8 — Validacion cruzada entre mercancia recibida, pedido y documentos del proveedor
+COM-Alm-1.9 — Confirmacion y registro de entrada de mercancia en el sistema</t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="2">
@@ -484,7 +504,8 @@
       </c>
       <c r="I6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COC-4.4, COC-4.6</t>
+          <t xml:space="preserve">COC-4.4 — Entrega de productos desde almacen y firma de entrega
+COC-4.6 — Notificacion a Gerencia de reabastecimiento de agua potable y gas</t>
         </is>
       </c>
       <c r="J6" t="inlineStr" s="2">
@@ -494,17 +515,21 @@
       </c>
       <c r="K6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-3.7, AFJ-7.1, AFJ-7.2, AFJ-7.5</t>
+          <t xml:space="preserve">AFJ-3.7 — Supervision de pedidos recibidos en Almacen con respaldo documental
+AFJ-7.1 — Atencion a proveedores en despachos (agua, gas, Internet)
+AFJ-7.2 — Supervision de recepcion de pedidos de gran envergadura
+AFJ-7.5 — Recepcion de mercancias/equipos no almacenables en administracion</t>
         </is>
       </c>
       <c r="L6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-14.2</t>
+          <t xml:space="preserve">AFL-14.2 — Recepcion fisica y en Odoo de pedidos</t>
         </is>
       </c>
       <c r="M6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-3.1, GHO-3.2</t>
+          <t xml:space="preserve">GHO-3.1 — Gestion y solicitud de suministro de agua potable
+GHO-3.2 — Solicitud de llenado de tanques de gas</t>
         </is>
       </c>
       <c r="N6" t="inlineStr" s="2">
@@ -531,7 +556,7 @@
       </c>
       <c r="D7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COM-Alm-1.11</t>
+          <t xml:space="preserve">COM-Alm-1.11 — Despacho de mercancia a departamentos internos contra requisicion escrita</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="2">
@@ -546,12 +571,13 @@
       </c>
       <c r="G7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CAJ-1.5, CAJ-3.5</t>
+          <t xml:space="preserve">CAJ-1.5 — Reposicion de productos para nevera y vitrina en el almacen de caja
+CAJ-3.5 — Retiro de productos solicitados y almacenamiento en el almacen de caja</t>
         </is>
       </c>
       <c r="H7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">BAR-4.4</t>
+          <t xml:space="preserve">BAR-4.4 — Entrega de productos desde almacen y firma de entrega</t>
         </is>
       </c>
       <c r="I7" t="inlineStr" s="2">
@@ -566,7 +592,7 @@
       </c>
       <c r="K7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-7.3</t>
+          <t xml:space="preserve">AFJ-7.3 — Ordenes de entrada y salida de productos, mercancia, articulos</t>
         </is>
       </c>
       <c r="L7" t="inlineStr" s="2">
@@ -581,7 +607,7 @@
       </c>
       <c r="N7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OPE-3.5</t>
+          <t xml:space="preserve">OPE-3.5 — Entrega de herramientas y materiales desde el taller</t>
         </is>
       </c>
     </row>
@@ -603,7 +629,7 @@
       </c>
       <c r="D8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COM-Alm-1.10</t>
+          <t xml:space="preserve">COM-Alm-1.10 — Ubicacion fisica de mercancia recepcionada en el almacen</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="2">
@@ -685,22 +711,36 @@
       </c>
       <c r="F9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CTR-3.1, CTR-3.2, CTR-3.3, CTR-7.1</t>
+          <t xml:space="preserve">CTR-3.1 — Coordinacion de inventario ciclico diario con encargado de almacen
+CTR-3.2 — Verificacion en sistema de existencias y movimientos de productos
+CTR-3.3 — Depuracion integral del inventario para entrega a responsable administrativo
+CTR-7.1 — Descarga de reportes de inventario desde Odoo</t>
         </is>
       </c>
       <c r="G9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CAJ-1.3, CAJ-1.4, CAJ-1.6, CAJ-1.16, CAJ-3.1, CAJ-4.8</t>
+          <t xml:space="preserve">CAJ-1.3 — Inventario ciclico para reposicion de productos en la nevera
+CAJ-1.4 — Inventario ciclico para reposicion de productos en la vitrina
+CAJ-1.6 — Firma de ficha de reposicion de productos
+CAJ-1.16 — Verificacion de inventario, nevera y vitrina
+CAJ-3.1 — Inventario general
+CAJ-4.8 — Inventario de productos (turno tarde)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">BAR-2.2, BAR-2.11, BAR-4.1</t>
+          <t xml:space="preserve">BAR-2.2 — Inventario de productos y mise en place de suministros y materiales
+BAR-2.11 — Inventario de plateria y manteleria
+BAR-4.1 — Inventario diario/manual del area</t>
         </is>
       </c>
       <c r="I9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COC-1.3, COC-2.2, COC-3.1, COC-4.1, COC-5.1</t>
+          <t xml:space="preserve">COC-1.3 — Verificacion de productos/insumos para el desayuno
+COC-2.2 — Verificacion de productos/insumos para almuerzo
+COC-3.1 — Inventario de productos para snacks
+COC-4.1 — Inventario diario/manual en el almacen de cocina
+COC-5.1 — Inventario de productos para cena</t>
         </is>
       </c>
       <c r="J9" t="inlineStr" s="2">
@@ -710,17 +750,18 @@
       </c>
       <c r="K9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-7.9</t>
+          <t xml:space="preserve">AFJ-7.9 — Apoyo en la realizacion de inventarios generales o departamentales</t>
         </is>
       </c>
       <c r="L9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-15.1</t>
+          <t xml:space="preserve">AFL-15.1 — Supervision aleatoria de inventarios en almacenes</t>
         </is>
       </c>
       <c r="M9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-1.4.1, GHO-1.4.4</t>
+          <t xml:space="preserve">GHO-1.4.1 — Inventario mensual de mercancia (Mambo y Playera)
+GHO-1.4.4 — Registro de movimientos de inventario en Cloudbeds</t>
         </is>
       </c>
       <c r="N9" t="inlineStr" s="2">
@@ -767,7 +808,8 @@
       </c>
       <c r="H10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">BAR-1.5, BAR-3.4</t>
+          <t xml:space="preserve">BAR-1.5 — Verificacion de productos a servir
+BAR-3.4 — Verificacion de productos a servir (cena)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr" s="2">
@@ -834,17 +876,46 @@
       </c>
       <c r="G11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CAJ-1.7, CAJ-1.8, CAJ-1.9, CAJ-1.10, CAJ-1.11, CAJ-1.15, CAJ-4.1, CAJ-4.2, CAJ-4.3, CAJ-4.4, CAJ-4.5, CAJ-2.8</t>
+          <t xml:space="preserve">CAJ-1.7 — Conteo de desayuno por habitacion
+CAJ-1.8 — Asignacion de numero de mesa al huesped
+CAJ-1.9 — Creacion de comanda en Poster (habitacion, mesa, pedido)
+CAJ-1.10 — Impresion de comandas para cocina y barra
+CAJ-1.11 — Impresion de comanda general por habitacion
+CAJ-1.15 — Determinar huespedes faltantes por comer
+CAJ-4.1 — Recepcion del pedido de huesped
+CAJ-4.2 — Creacion de comanda en Poster (habitacion, nombre, pedido)
+CAJ-4.3 — Confirmacion con el mesonero
+CAJ-4.4 — Impresion de comanda para cocina/barra/snacks
+CAJ-4.5 — Verificacion del pedido
+CAJ-2.8 — Impresion de recibo de hielo para huesped</t>
         </is>
       </c>
       <c r="H11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">BAR-1.6, BAR-1.7, BAR-1.8, BAR-1.9, BAR-1.10, BAR-2.4, BAR-2.5, BAR-2.6, BAR-2.7, BAR-2.8, BAR-3.5, BAR-3.6, BAR-3.7, BAR-3.8, BAR-3.9</t>
+          <t xml:space="preserve">BAR-1.6 — Toma de pedido de huespedes (desayuno)
+BAR-1.7 — Entrega de comandas a Caja para enviar a Cocina (desayuno)
+BAR-1.8 — Verificar que el pedido haya llegado completo a cocina (desayuno)
+BAR-1.9 — Preparacion del pedido (desayuno)
+BAR-1.10 — Entrega al comensal (desayuno)
+BAR-2.4 — Toma de pedido de huespedes (almuerzo esporadico)
+BAR-2.5 — Entrega de comandas a Caja para enviar a Cocina (almuerzo)
+BAR-2.6 — Verificar que el pedido haya llegado completo a cocina (almuerzo)
+BAR-2.7 — Preparacion del pedido (almuerzo)
+BAR-2.8 — Entrega al comensal (almuerzo)
+BAR-3.5 — Toma de pedido de huespedes (snack/cena)
+BAR-3.6 — Entrega de comandas a Caja para enviar a Cocina (cena)
+BAR-3.7 — Verificar que el pedido haya llegado completo a cocina (cena)
+BAR-3.8 — Preparacion del pedido (cena)
+BAR-3.9 — Entrega al comensal (cena)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COC-2.4, COC-3.3, COC-5.4, COC-3.4, COC-2.5</t>
+          <t xml:space="preserve">COC-2.4 — Recepcion de pedidos de huespedes (almuerzo)
+COC-3.3 — Recepcion de pedidos de huespedes (snacks/cena)
+COC-5.4 — Cena de huespedes
+COC-3.4 — Snacks para huespedes
+COC-2.5 — Almuerzos de huespedes</t>
         </is>
       </c>
       <c r="J11" t="inlineStr" s="2">
@@ -906,12 +977,14 @@
       </c>
       <c r="G12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CAJ-4.0, CAJ-1.12</t>
+          <t xml:space="preserve">CAJ-4.0 — Entrega de guardia de turno (3:00 PM)
+CAJ-1.12 — Recoleccion de firma de huesped</t>
         </is>
       </c>
       <c r="H12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">BAR-2.10, BAR-3.11</t>
+          <t xml:space="preserve">BAR-2.10 — Entrega de guardia de turno (manana a tarde)
+BAR-3.11 — Entrega de guardia de turno (tarde a manana, con inventario de cierre)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr" s="2">
@@ -978,7 +1051,13 @@
       </c>
       <c r="G13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CAJ-1.13, CAJ-1.14, CAJ-1.18, CAJ-4.7, CAJ-2.6, CAJ-2.5, CAJ-4.6</t>
+          <t xml:space="preserve">CAJ-1.13 — Envio de comandas a recepcion desde Poster
+CAJ-1.14 — Envio de comanda firmada por huesped a recepcion
+CAJ-1.18 — Verificacion de dia de check-out de huesped
+CAJ-4.7 — Envio de comandas a recepcion desde Poster (turno tarde)
+CAJ-2.6 — Envio de comanda firmada por huesped a recepcion
+CAJ-2.5 — Recoleccion de firma de huesped para la comanda de cava
+CAJ-4.6 — Recoleccion de firma de huesped para la comanda</t>
         </is>
       </c>
       <c r="H13" t="inlineStr" s="2">
@@ -1008,7 +1087,7 @@
       </c>
       <c r="M13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-1.2.1</t>
+          <t xml:space="preserve">GHO-1.2.1 — Gestion de cobros de consumos y servicios adicionales</t>
         </is>
       </c>
       <c r="N13" t="inlineStr" s="2">
@@ -1060,7 +1139,10 @@
       </c>
       <c r="I14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COC-1.2, COC-2.3, COC-3.2, COC-5.2</t>
+          <t xml:space="preserve">COC-1.2 — Mise en place de productos y utensilios (desayuno)
+COC-2.3 — Mise en place de productos y utensilios (almuerzo)
+COC-3.2 — Mise en place de productos y utensilios (snacks)
+COC-5.2 — Mise en place de productos y utensilios (cena)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr" s="2">
@@ -1132,7 +1214,10 @@
       </c>
       <c r="I15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COC-7.1, COC-7.2, COC-7.3, COC-7.4</t>
+          <t xml:space="preserve">COC-7.1 — Limpiezas de proteinas (carne, pollo, mariscos y pescado)
+COC-7.2 — Pesos de proteinas
+COC-7.3 — Embolsado de proteinas
+COC-7.4 — Inventario de lo que se saca (conteo)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr" s="2">
@@ -1194,7 +1279,11 @@
       </c>
       <c r="G16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CAJ-2.1, CAJ-2.2, CAJ-2.3, CAJ-2.4, CAJ-2.7</t>
+          <t xml:space="preserve">CAJ-2.1 — Asignacion de cava para el huesped
+CAJ-2.2 — Solicitud de firma de huesped para cava
+CAJ-2.3 — Identificacion de huesped para la cava
+CAJ-2.4 — Recepcion de pedido para cava en Poster
+CAJ-2.7 — Crear el listado de cavas por huesped</t>
         </is>
       </c>
       <c r="H16" t="inlineStr" s="2">
@@ -1291,12 +1380,26 @@
       </c>
       <c r="L17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-1.2, AFL-1.3, AFL-1.4, AFL-1.5, AFL-1.6, AFL-3.2, AFL-3.3, AFL-3.4, AFL-3.5, AFL-3.6, AFL-5.2, AFL-5.3, AFL-5.4, AFL-8.1, AFL-8.2</t>
+          <t xml:space="preserve">AFL-1.2 — Exportacion y validacion del informe de caja desde Cloudbeds
+AFL-1.3 — Recepcion fisica del efectivo al cierre de turno de recepcion
+AFL-1.4 — Conciliacion del efectivo entregado contra registros de Cloudbeds
+AFL-1.5 — Registro del efectivo del cierre en los diarios de caja de Odoo
+AFL-1.6 — Exportacion del informe de conciliacion de pagos desde Cloudbeds
+AFL-3.2 — Exportacion del informe de turno de caja desde Poster
+AFL-3.3 — Recepcion fisica del efectivo del cierre de turno de A&amp;B
+AFL-3.4 — Conciliacion del efectivo de A&amp;B contra registros de Poster
+AFL-3.5 — Registro contable del efectivo de A&amp;B en diarios de caja
+AFL-3.6 — Exportacion del informe de recibos desde Poster
+AFL-5.2 — Recepcion del reporte fisico de estacionamiento
+AFL-5.3 — Elaboracion y envio del reporte de cierre de estacionamiento
+AFL-5.4 — Registro en Odoo de los pagos de estacionamiento
+AFL-8.1 — Recepcion y resguardo del efectivo en la caja principal
+AFL-8.2 — Registro contable de movimientos de la caja principal en Odoo</t>
         </is>
       </c>
       <c r="M17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-1.1.7</t>
+          <t xml:space="preserve">GHO-1.1.7 — Ejecucion de cierres de turnos</t>
         </is>
       </c>
       <c r="N17" t="inlineStr" s="2">
@@ -1363,12 +1466,38 @@
       </c>
       <c r="L18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-1.1, AFL-1.7, AFL-1.8, AFL-3.1, AFL-3.7, AFL-3.8, AFL-4.1, AFL-4.2, AFL-5.1, AFL-6.1, AFL-6.2, AFL-6.3, AFL-6.4, AFL-7.1, AFL-7.2, AFL-7.3, AFL-7.4, AFL-11.1, AFL-12.1</t>
+          <t xml:space="preserve">AFL-1.1 — Verificacion de pagos bancarios y confirmacion a recepcion
+AFL-1.7 — Verificacion cruzada de pagos electronicos contra Cloudbeds y banco
+AFL-1.8 — Notificacion de errores a recepcion y gestion de anulaciones
+AFL-3.1 — Verificacion de pagos bancarios para la caja de A&amp;B
+AFL-3.7 — Conciliacion de pagos electronicos de A&amp;B contra banco y Poster
+AFL-3.8 — Gestion de errores en el cierre de A&amp;B (fe de errata)
+AFL-4.1 — Creacion del contacto del cliente en Odoo para A&amp;B
+AFL-4.2 — Registro de recibos de cobro y factura de consumos de A&amp;B
+AFL-5.1 — Verificacion de pagos bancarios para el cierre de estacionamiento
+AFL-6.1 — Recepcion y desglose del reporte semanal de traslados de la Marina
+AFL-6.2 — Confirmacion del pago de la Marina
+AFL-6.3 — Envio del reporte semanal de traslados a Administracion
+AFL-6.4 — Registro en Odoo del pago de traslados de la Marina
+AFL-7.1 — Recepcion y desglose del reporte semanal de Boca Seca
+AFL-7.2 — Confirmacion del pago de Boca Seca
+AFL-7.3 — Envio del reporte semanal de Boca Seca a Administracion
+AFL-7.4 — Registro en Odoo de pagos en efectivo de Boca Seca (NF)
+AFL-11.1 — Registro del recibo de cobro en efectivo en Odoo
+AFL-12.1 — Registro del recibo de cobro en divisas digitales</t>
         </is>
       </c>
       <c r="M18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-1.1.3, GHO-1.1.4, GHO-1.1.5, GHO-1.1.6, GHO-1.2.2, GHO-1.2.3, GHO-1.2.4, GHO-1.3.1, GHO-1.3.2</t>
+          <t xml:space="preserve">GHO-1.1.3 — Gestion de cobros multimedia
+GHO-1.1.4 — Carga y conciliacion de pagos en Cloudbeds
+GHO-1.1.5 — Carga de registros contables en Odoo
+GHO-1.1.6 — Anexo y reporte de ingresos en Microsoft Teams
+GHO-1.2.2 — Carga y conciliacion de pagos de check-out en Cloudbeds
+GHO-1.2.3 — Carga de registros contables de salida en Odoo
+GHO-1.2.4 — Anexo y reporte de ingresos de check-out en Teams
+GHO-1.3.1 — Envio de comprobantes de pagos a Administracion
+GHO-1.3.2 — Confirmacion de pagos a los huespedes por correo</t>
         </is>
       </c>
       <c r="N18" t="inlineStr" s="2">
@@ -1400,7 +1529,7 @@
       </c>
       <c r="E19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-2.4.1</t>
+          <t xml:space="preserve">RRH-2.4.1 — Conciliacion en Odoo de movimientos vinculados a pagos</t>
         </is>
       </c>
       <c r="F19" t="inlineStr" s="2">
@@ -1425,17 +1554,23 @@
       </c>
       <c r="J19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.1.1, CCS-4.1.3, CCS-4.1.7, CCS-4.1.8</t>
+          <t xml:space="preserve">CCS-4.1.1 — Disponibilidad diaria (antes de las 10:30 am)
+CCS-4.1.3 — Seguimiento a las tasas bancarias
+CCS-4.1.7 — Carga de extracto bancario luego de las 10:30 am
+CCS-4.1.8 — Carga y cotejo del estado de cuenta bancario y caja</t>
         </is>
       </c>
       <c r="K19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-1.10, AFJ-1.11</t>
+          <t xml:space="preserve">AFJ-1.10 — Conciliacion de pagos y cierre de factura
+AFJ-1.11 — Archivo de pagos por origen bancario con su comprobante en la nube</t>
         </is>
       </c>
       <c r="L19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-10.1, AFL-10.2, AFL-10.3</t>
+          <t xml:space="preserve">AFL-10.1 — Descarga del extracto bancario de cada banco
+AFL-10.2 — Descarga del detalle de lotes de POS desde Credicard
+AFL-10.3 — Conciliacion bancaria cruzando recibos con extractos</t>
         </is>
       </c>
       <c r="M19" t="inlineStr" s="2">
@@ -1507,7 +1642,11 @@
       </c>
       <c r="L20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-8.5, AFL-11.2, AFL-11.3, AFL-12.2, AFL-12.3</t>
+          <t xml:space="preserve">AFL-8.5 — Conciliacion de la caja principal (remite a Area 11)
+AFL-11.2 — Creacion manual del extracto de caja en Odoo
+AFL-11.3 — Conciliacion de recibos en efectivo contra extracto de caja
+AFL-12.2 — Creacion manual del extracto de divisas en Odoo
+AFL-12.3 — Conciliacion de recibos en divisas contra extracto</t>
         </is>
       </c>
       <c r="M20" t="inlineStr" s="2">
@@ -1579,7 +1718,16 @@
       </c>
       <c r="L21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-2.1, AFL-2.2, AFL-2.3, AFL-2.4, AFL-2.5, AFL-4.3, AFL-5.5, AFL-6.5, AFL-16.1, AFL-16.2</t>
+          <t xml:space="preserve">AFL-2.1 — Revision de la cuenta del cliente en Cloudbeds previo a facturar
+AFL-2.2 — Validacion del contacto del cliente en Odoo previo a facturar
+AFL-2.3 — Validacion de los recibos de cobro del cliente en Odoo
+AFL-2.4 — Creacion de la factura de venta en Odoo
+AFL-2.5 — Impresion de la factura de contingencia
+AFL-4.3 — Impresion de la factura de contingencia de A&amp;B
+AFL-5.5 — Impresion de la factura de contingencia de estacionamiento
+AFL-6.5 — Impresion de la factura de contingencia de la Marina
+AFL-16.1 — Gestion de cobro a arrendatarios y emision de factura
+AFL-16.2 — Emision de factura de arrendamiento en Odoo</t>
         </is>
       </c>
       <c r="M21" t="inlineStr" s="2">
@@ -1651,12 +1799,17 @@
       </c>
       <c r="L22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-13.6, AFL-13.9</t>
+          <t xml:space="preserve">AFL-13.6 — Actualizacion de precios de productos en Poster
+AFL-13.9 — Diseno e impresion del menu fisico de A&amp;B en Canva</t>
         </is>
       </c>
       <c r="M22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-2.2.1, GHO-2.2.2, GHO-2.2.3, GHO-2.2.4, GHO-2.3.3</t>
+          <t xml:space="preserve">GHO-2.2.1 — Gestion de cuentas de agencias de viajes y operadores
+GHO-2.2.2 — Coordinacion de grupos y eventos
+GHO-2.2.3 — Protocolo de atencion a clientes VIP
+GHO-2.2.4 — Atencion a agentes gubernamentales
+GHO-2.3.3 — Aplicacion y autorizacion de descuentos especiales</t>
         </is>
       </c>
       <c r="N22" t="inlineStr" s="2">
@@ -1683,7 +1836,7 @@
       </c>
       <c r="D23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COM-2</t>
+          <t xml:space="preserve">COM-2 — Revision y cierre quincenal de pedidos</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="2">
@@ -1713,12 +1866,20 @@
       </c>
       <c r="J23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.1.2</t>
+          <t xml:space="preserve">CCS-4.1.2 — Planificacion de pagos (proveedores, gubernamental, municipal)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-3.1, AFJ-3.2, AFJ-3.3, AFJ-3.4, AFJ-3.5, AFJ-3.6, AFJ-3.8, AFJ-3.9, AFJ-3.10</t>
+          <t xml:space="preserve">AFJ-3.1 — Verificacion de pedidos de proveedores con ventas a credito
+AFJ-3.2 — Organizar manualmente los pedidos para totalizar en archivo
+AFJ-3.3 — Reporte diario de actualizacion de cuentas por pagar
+AFJ-3.4 — Marcar facturas pagadas/pendientes con tutoria de Gerencia de Finanzas
+AFJ-3.5 — Validacion de cuentas por pagar vencidas en plazos de credito
+AFJ-3.6 — Registro y archivo de notas de despacho de cuentas por pagar
+AFJ-3.8 — Comunicacion con proveedores sobre pagos, solvencias y comprobantes
+AFJ-3.9 — Actualizacion manual de CxP de proveedores con factura directa
+AFJ-3.10 — Inclusion manual de servicios mensuales (CORPOELEC/TELMACA/seguridad)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr" s="2">
@@ -1755,7 +1916,7 @@
       </c>
       <c r="D24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COM-1.4</t>
+          <t xml:space="preserve">COM-1.4 — Solicitud y gestion de documentos al proveedor segun condicion de pago</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="2">
@@ -1785,27 +1946,40 @@
       </c>
       <c r="J24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.2.1, CCS-4.2.3, CCS-4.2.5, CCS-4.2.6, CCS-4.2.8, CCS-4.1.9, CCS-4.1.10</t>
+          <t xml:space="preserve">CCS-4.2.1 — Pago a proveedores verificando pedido autorizado
+CCS-4.2.3 — Pago mensual de 23 tarjetas Simple TV
+CCS-4.2.5 — Recarga de combustible semanal (chofer de presidencia)
+CCS-4.2.6 — Pago de combustible Tiggo Pro8
+CCS-4.2.8 — Pago Corpoelec Dr. Acid Margarita + Prados del Este
+CCS-4.1.9 — Transferencias por propina, vuelto o error
+CCS-4.1.10 — Recarga de Cobre TAG (pago de presidencia)</t>
         </is>
       </c>
       <c r="K24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-1.1, AFJ-1.3, AFJ-1.4, AFJ-1.5, AFJ-1.7, AFJ-1.8, AFJ-1.9</t>
+          <t xml:space="preserve">AFJ-1.1 — Verificacion y validacion del documento antes de procesarlo
+AFJ-1.3 — Verificacion y validacion del pedido antes de importarlo a la factura
+AFJ-1.4 — Solicitud de facturas a proveedores (chat directo)
+AFJ-1.5 — Registro de facturas
+AFJ-1.7 — Solicitud de pago a Finanzas
+AFJ-1.8 — Emision de pagos de facturas a proveedores (envio de comprobante)
+AFJ-1.9 — Aplicacion de pago a la factura</t>
         </is>
       </c>
       <c r="L24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-8.3, AFL-8.4</t>
+          <t xml:space="preserve">AFL-8.3 — Pago a proveedores desde la caja principal con autorizacion
+AFL-8.4 — Pago a empleados desde la caja principal con autorizacion</t>
         </is>
       </c>
       <c r="M24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-3.4</t>
+          <t xml:space="preserve">GHO-3.4 — Firma de pedidos extraordinarios en ausencia de Gerencia General</t>
         </is>
       </c>
       <c r="N24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OPE-5.2</t>
+          <t xml:space="preserve">OPE-5.2 — Llenado de tanque de agua</t>
         </is>
       </c>
     </row>
@@ -1862,7 +2036,8 @@
       </c>
       <c r="K25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-1.18, AFJ-1.19</t>
+          <t xml:space="preserve">AFJ-1.18 — Facturacion de proveedores pagados sin factura y encuadre de anticipos
+AFJ-1.19 — Validacion y aplicacion/depuracion de anticipos de proveedores</t>
         </is>
       </c>
       <c r="L25" t="inlineStr" s="2">
@@ -1929,7 +2104,10 @@
       </c>
       <c r="J26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.4.4, CCS-4.2.7, CCS-4.2.9, CCS-4.2.10</t>
+          <t xml:space="preserve">CCS-4.4.4 — Asientos contables en facturas de compra para CxP socios Racid
+CCS-4.2.7 — Pago de arrendamiento Dr. Acid Margarita (CxC socio)
+CCS-4.2.9 — Relacion de CxP de arrendamiento piso 4
+CCS-4.2.10 — Pago del VACC (CxC socios Racid)</t>
         </is>
       </c>
       <c r="K26" t="inlineStr" s="2">
@@ -2001,7 +2179,7 @@
       </c>
       <c r="J27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.4.8</t>
+          <t xml:space="preserve">CCS-4.4.8 — Devoluciones en Odoo por error</t>
         </is>
       </c>
       <c r="K27" t="inlineStr" s="2">
@@ -2043,12 +2221,13 @@
       </c>
       <c r="D28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COM-3</t>
+          <t xml:space="preserve">COM-3 — Gestion de reembolsos de IVA e ISLR con proveedores</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-2.6.1, RRH-2.6.2</t>
+          <t xml:space="preserve">RRH-2.6.1 — Elaboracion de archivo XML para declaracion de retenciones ISLR
+RRH-2.6.2 — Elaboracion mensual de hoja de trabajo para la contribucion DPP</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="2">
@@ -2073,17 +2252,22 @@
       </c>
       <c r="J28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.3.1, CCS-4.3.2, CCS-4.4.7, CCS-4.2.2</t>
+          <t xml:space="preserve">CCS-4.3.1 — Revisar XML + TXT por inconsistencias (declaracion quincenal)
+CCS-4.3.2 — Generar y fusionar XML de retencion de sueldos y salarios
+CCS-4.4.7 — Verificacion de aplicacion de ISLR en lineas de factura
+CCS-4.2.2 — Solicitar reembolso de retenciones a proveedores</t>
         </is>
       </c>
       <c r="K28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-2.6, AFJ-3.11</t>
+          <t xml:space="preserve">AFJ-2.6 — Revision y validacion de retenciones IVA/ISLR del periodo
+AFJ-3.11 — Emision y archivo de certificados de retencion</t>
         </is>
       </c>
       <c r="L28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-17.1, AFL-17.2</t>
+          <t xml:space="preserve">AFL-17.1 — Registro de comprobantes de retencion de IVA en Odoo
+AFL-17.2 — Registro de comprobantes de retencion de ISLR en Odoo</t>
         </is>
       </c>
       <c r="M28" t="inlineStr" s="2">
@@ -2125,7 +2309,8 @@
       </c>
       <c r="F29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CTR-5.2, CTR-7.2</t>
+          <t xml:space="preserve">CTR-5.2 — Auditoria de movimientos fiscales
+CTR-7.2 — Descarga de libros contables desde Odoo</t>
         </is>
       </c>
       <c r="G29" t="inlineStr" s="2">
@@ -2150,7 +2335,11 @@
       </c>
       <c r="K29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-2.1, AFJ-2.2, AFJ-2.3, AFJ-2.5, AFJ-2.7</t>
+          <t xml:space="preserve">AFJ-2.1 — Informar el cese de registro de facturas e iniciar el descargue del libro
+AFJ-2.2 — Verificacion en 1era revision de documentos a declarar
+AFJ-2.3 — Verificacion y conteo de documentos archivados Tucacas/Caracas
+AFJ-2.5 — Validar el cierre total de las facturas a declarar
+AFJ-2.7 — Enumeracion del libro de compras en la nube</t>
         </is>
       </c>
       <c r="L29" t="inlineStr" s="2">
@@ -2197,7 +2386,8 @@
       </c>
       <c r="F30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CTR-1.2, CTR-1.3</t>
+          <t xml:space="preserve">CTR-1.2 — Monitoreo y seguimiento de operaciones
+CTR-1.3 — Analisis mensual de informacion financiera</t>
         </is>
       </c>
       <c r="G30" t="inlineStr" s="2">
@@ -2289,7 +2479,11 @@
       </c>
       <c r="J31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.3.6, CCS-4.3.7, CCS-4.3.8, CCS-4.3.9, CCS-4.3.10</t>
+          <t xml:space="preserve">CCS-4.3.6 — Pago mensual de FONACIT (0,50%)
+CCS-4.3.7 — Pago mensual de INATUR (1%)
+CCS-4.3.8 — Pago mensual ante Alcaldia Municipio Silva (2%)
+CCS-4.3.9 — Pago mensual de INPARQUES
+CCS-4.3.10 — Pago mensual de aseo urbano (ISMA)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr" s="2">
@@ -2336,7 +2530,12 @@
       </c>
       <c r="E32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-1.1.1, RRH-1.1.2, RRH-1.1.3, RRH-1.1.4, RRH-3.6.3, RRH-3.6.4</t>
+          <t xml:space="preserve">RRH-1.1.1 — Revision mensual de documentacion de IVSS, INCES, FAOV y MPPPST
+RRH-1.1.2 — Listado de personal activo, estados de cuenta y solvencias
+RRH-1.1.3 — Reporte de compromisos y seguimiento de pagos a Administracion y Finanzas
+RRH-1.1.4 — Actualizacion mensual de la carpeta Oslo con informacion parafiscal
+RRH-3.6.3 — Preparacion de ARC (Comprobante de Agente de Retencion)
+RRH-3.6.4 — Preparacion de ARI (Ajuste de Retenciones de ISLR)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="2">
@@ -2361,7 +2560,9 @@
       </c>
       <c r="J32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.3.3, CCS-4.3.4, CCS-4.3.5</t>
+          <t xml:space="preserve">CCS-4.3.3 — Revision y envio mensual del IPP de trabajadores
+CCS-4.3.4 — Preparacion de informacion para declaracion anual de ISLR
+CCS-4.3.5 — Preparacion de informacion para declaracion de IGP</t>
         </is>
       </c>
       <c r="K32" t="inlineStr" s="2">
@@ -2408,12 +2609,15 @@
       </c>
       <c r="E33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-1.2.1/1.2.2, RRH-1.2.3, RRH-3.6.5</t>
+          <t xml:space="preserve">RRH-1.2.1/1.2.2 — Solicitud y revision de documentacion de SENIAT, INATUR, Alcaldia, Bomberos, MINTUR, RUPDAE y LOCTI
+RRH-1.2.3 — Atencion a entes gubernamentales y soporte en auditorias
+RRH-3.6.5 — Emision de constancias de trabajo, 14-100, 14-02, certificados IVSS y FAOV</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CTR-5.1, CTR-5.3</t>
+          <t xml:space="preserve">CTR-5.1 — Coordinacion de auditorias y envio de informacion a asesor contable externo
+CTR-5.3 — Organizacion preventiva de documentacion para fiscalizaciones</t>
         </is>
       </c>
       <c r="G33" t="inlineStr" s="2">
@@ -2433,12 +2637,16 @@
       </c>
       <c r="J33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.4.3, CCS-4.4.9</t>
+          <t xml:space="preserve">CCS-4.4.3 — Vinculacion de facturas escaneadas en Odoo (cierre)
+CCS-4.4.9 — Archivo y orden de facturas fiscales de compra y venta</t>
         </is>
       </c>
       <c r="K33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-1.12, AFJ-1.13, AFJ-1.14, AFJ-2.4</t>
+          <t xml:space="preserve">AFJ-1.12 — Escaneo e identificacion de documentos para el cierre fiscal
+AFJ-1.13 — Archivo y resguardo de documentos fisicos procesados
+AFJ-1.14 — Organizar, embalar y enviar valija a administracion Caracas
+AFJ-2.4 — Seguimiento de documentos en transito en manos de proveedores</t>
         </is>
       </c>
       <c r="L33" t="inlineStr" s="2">
@@ -2510,7 +2718,7 @@
       </c>
       <c r="K34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-1.6</t>
+          <t xml:space="preserve">AFJ-1.6 — Recepcion de guias SUNAGRO SICA</t>
         </is>
       </c>
       <c r="L34" t="inlineStr" s="2">
@@ -2552,7 +2760,15 @@
       </c>
       <c r="E35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-2.1.2, RRH-2.1.3, RRH-2.3.1, RRH-2.3.2, RRH-2.3.5, RRH-2.5.1, RRH-2.5.2, RRH-2.4.2, RRH-3.7.1</t>
+          <t xml:space="preserve">RRH-2.1.2 — Planificacion mensual y quincenal de pagos
+RRH-2.1.3 — Envio de prevision de fondos a Administracion y Finanzas
+RRH-2.3.1 — Calculo semanal de horas extras
+RRH-2.3.2 — Envio de reporte para aprobacion a Administracion y Finanzas
+RRH-2.3.5 — Gestion del bono de productividad a camareras
+RRH-2.5.1 — Registro quincenal de consumos internos del personal
+RRH-2.5.2 — Aplicacion de descuentos por consumos, ausencias, retardos y abonos a CxC
+RRH-2.4.2 — Actualizacion de estados de CxC por trabajador
+RRH-3.7.1 — Pago de liquidacion</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="2">
@@ -2624,7 +2840,8 @@
       </c>
       <c r="E36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-2.3.3, RRH-2.3.4</t>
+          <t xml:space="preserve">RRH-2.3.3 — Elaboracion de archivo masivo (TXT) para pago de horas extras y nomina
+RRH-2.3.4 — Transferencias individuales a colaboradores con cuentas de otros bancos</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="2">
@@ -2696,7 +2913,9 @@
       </c>
       <c r="E37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-2.2.1, RRH-2.2.2, RRH-2.2.3</t>
+          <t xml:space="preserve">RRH-2.2.1 — Registro diario de asistencia del personal
+RRH-2.2.2 — Revision diaria de retardos y ausencias justificadas e injustificadas
+RRH-2.2.3 — Recepcion y validacion de horas extras por departamento</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="2">
@@ -2736,7 +2955,7 @@
       </c>
       <c r="M37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-2.4.4</t>
+          <t xml:space="preserve">GHO-2.4.4 — Control de redobles y gestion de dias libres trabajados</t>
         </is>
       </c>
       <c r="N37" t="inlineStr" s="2">
@@ -2768,7 +2987,11 @@
       </c>
       <c r="E38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-3.1.1, RRH-3.1.2, RRH-3.1.3, RRH-3.1.4, RRH-3.1.5</t>
+          <t xml:space="preserve">RRH-3.1.1 — Elaboracion de flyers de vacantes
+RRH-3.1.2 — Publicacion de vacantes en WhatsApp, Telegram y grupos operativos
+RRH-3.1.3 — Preseleccion, filtros, entrevistas y aplicacion de pruebas
+RRH-3.1.4 — Entrega y recepcion de kit de reclutamiento
+RRH-3.1.5 — Presentacion final de candidatos a Gerencia General</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="2">
@@ -2808,7 +3031,7 @@
       </c>
       <c r="M38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-2.4.5</t>
+          <t xml:space="preserve">GHO-2.4.5 — Analisis de perfiles para reclutamiento de recepcion</t>
         </is>
       </c>
       <c r="N38" t="inlineStr" s="2">
@@ -2840,7 +3063,13 @@
       </c>
       <c r="E39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-3.2.2, RRH-3.2.4, RRH-3.3.1, RRH-3.3.2, RRH-3.3.3, RRH-3.3.4, RRH-3.3.5</t>
+          <t xml:space="preserve">RRH-3.2.2 — Creacion de empleado en Odoo
+RRH-3.2.4 — Entrega de tarjeta bancaria y activacion del kit nomina
+RRH-3.3.1 — Actualizacion permanente de base de datos de personal
+RRH-3.3.2 — Mantenimiento de expedientes fisicos y digitales
+RRH-3.3.3 — Levantamiento de informacion para descripciones de cargo
+RRH-3.3.4 — Actualizacion de organigrama
+RRH-3.3.5 — Registro fotografico del personal</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="2">
@@ -2912,7 +3141,11 @@
       </c>
       <c r="E40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-3.2.1, RRH-3.2.3, RRH-3.7.2, RRH-3.7.3, RRH-3.7.4</t>
+          <t xml:space="preserve">RRH-3.2.1 — Solicitud de contrato al Departamento Legal
+RRH-3.2.3 — Induccion general y recorrido por las instalaciones
+RRH-3.7.2 — Entrega de kit de egreso
+RRH-3.7.3 — Recepcion de uniformes
+RRH-3.7.4 — Cierre de proceso por correo con documentacion digital</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="2">
@@ -2984,7 +3217,11 @@
       </c>
       <c r="E41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-3.4.1, RRH-3.4.2, RRH-3.4.4, RRH-3.4.5, RRH-3.5.1</t>
+          <t xml:space="preserve">RRH-3.4.1 — Revision semanal de horarios del personal
+RRH-3.4.2 — Coordinacion de dias libres del personal administrativo que pernocta
+RRH-3.4.4 — Gestion de solicitudes del personal (prestamos, vacaciones, adelantos, constancias)
+RRH-3.4.5 — Entrega y control de planillas de vacaciones
+RRH-3.5.1 — Atencion de solicitudes, permisos, reposos y certificados medicos (Forma 14-73)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="2">
@@ -3024,7 +3261,8 @@
       </c>
       <c r="M41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-2.4.1, GHO-2.4.3</t>
+          <t xml:space="preserve">GHO-2.4.1 — Elaboracion de horarios del departamento
+GHO-2.4.3 — Planificacion estrategica de equipos para temporadas altas</t>
         </is>
       </c>
       <c r="N41" t="inlineStr" s="2">
@@ -3056,7 +3294,7 @@
       </c>
       <c r="E42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-3.6.1</t>
+          <t xml:space="preserve">RRH-3.6.1 — Analisis de indicadores y ejecucion de la evaluacion de desempeno</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="2">
@@ -3128,7 +3366,8 @@
       </c>
       <c r="E43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-3.8.1, RRH-3.8.2</t>
+          <t xml:space="preserve">RRH-3.8.1 — Inventario y control de uniformes
+RRH-3.8.2 — Entrega de dotacion de equipos</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="2">
@@ -3158,7 +3397,10 @@
       </c>
       <c r="K43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-7.6, AFJ-7.7, AFJ-7.8, AFJ-7.10</t>
+          <t xml:space="preserve">AFJ-7.6 — Resguardo de llaves en la oficina de administracion
+AFJ-7.7 — Resguardo de material y equipo asignado por Gerencia General
+AFJ-7.8 — Entrega de equipos danados al Departamento de Tecnologia
+AFJ-7.10 — Distribucion enlistada de uniformes, materiales y equipos</t>
         </is>
       </c>
       <c r="L43" t="inlineStr" s="2">
@@ -3200,7 +3442,8 @@
       </c>
       <c r="E44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-1.3.1, RRH-1.3.2</t>
+          <t xml:space="preserve">RRH-1.3.1 — Verificacion mensual del Certificado de Manipulacion de Alimentos
+RRH-1.3.2 — Control mensual de vencimiento del Certificado de Salud</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="2">
@@ -3272,7 +3515,12 @@
       </c>
       <c r="E45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-4.1.1, RRH-4.1.3, RRH-4.1.4/4.1.5, RRH-4.1.7, RRH-4.1.8, RRH-4.1.9/4.1.10</t>
+          <t xml:space="preserve">RRH-4.1.1 — Entrevistas con universidades y solicitud de documentacion
+RRH-4.1.3 — Elaboracion de data y reporte a Gerencia General
+RRH-4.1.4/4.1.5 — Coordinacion de pernocta y recepcion y bienvenida de pasantes
+RRH-4.1.7 — Elaboracion de horarios semanales de pasantes
+RRH-4.1.8 — Mantenimiento de expediente fisico de pasantes
+RRH-4.1.9/4.1.10 — Evaluacion final, carta de culminacion y reporte a la coordinacion universitaria</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="2">
@@ -3344,7 +3592,7 @@
       </c>
       <c r="E46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-5.2</t>
+          <t xml:space="preserve">RRH-5.2 — Seguimiento de politicas de Seguridad y Salud en el Trabajo</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="2">
@@ -3416,7 +3664,13 @@
       </c>
       <c r="E47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">RRH-3.4.3, RRH-3.4.6, RRH-3.5.2, RRH-3.5.4, RRH-5.1, RRH-5.3, RRH-5.4</t>
+          <t xml:space="preserve">RRH-3.4.3 — Publicacion de horario requerido por el Ministerio del Trabajo
+RRH-3.4.6 — Actualizacion del listado de cumpleanos y reporte mensual a Gerencia
+RRH-3.5.2 — Elaboracion de llamados de atencion y comunicaciones disciplinarias
+RRH-3.5.4 — Redaccion de informes requeridos por la Gerencia General
+RRH-5.1 — Organizacion de agasajos y actividades corporativas
+RRH-5.3 — Comunicacion interna
+RRH-5.4 — Reporte inmediato de incidencias relacionadas con el personal</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="2">
@@ -3528,7 +3782,15 @@
       </c>
       <c r="M48" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-1.1.1, GHO-1.1.2, GHO-2.1.4, GHO-2.1.6, GHO-2.1.7, GHO-2.1.8, GHO-2.3.1, GHO-4.2, GHO-4.3</t>
+          <t xml:space="preserve">GHO-1.1.1 — Check-in de los huespedes
+GHO-1.1.2 — Registro de datos de los huespedes en Cloudbeds
+GHO-2.1.4 — Elaboracion de cotizaciones y creacion de reservas
+GHO-2.1.6 — Verificar y actualizar disponibilidad de habitaciones
+GHO-2.1.7 — Soporte en elaboracion de ingresos y ocupacion
+GHO-2.1.8 — Apoyar en el registro de huespedes
+GHO-2.3.1 — Acompanamiento a conocer las instalaciones
+GHO-4.2 — Verificacion y actualizacion de disponibilidad de habitaciones
+GHO-4.3 — Chequeo de habitaciones en mantenimiento para bloqueo/desbloqueo</t>
         </is>
       </c>
       <c r="N48" t="inlineStr" s="2">
@@ -3600,7 +3862,8 @@
       </c>
       <c r="M49" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-1.4.2, GHO-1.4.3</t>
+          <t xml:space="preserve">GHO-1.4.2 — Gestion y envio de pagos a los propietarios (cuentas externas)
+GHO-1.4.3 — Reporte a Talento Humano de ventas a empleados</t>
         </is>
       </c>
       <c r="N49" t="inlineStr" s="2">
@@ -3672,7 +3935,8 @@
       </c>
       <c r="M50" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-1.1.8, GHO-1.1.9</t>
+          <t xml:space="preserve">GHO-1.1.8 — Elaboracion de llaves electronicas de habitaciones
+GHO-1.1.9 — Realizacion de llaves maestras para ama de llaves, jefes y supervisores</t>
         </is>
       </c>
       <c r="N50" t="inlineStr" s="2">
@@ -3744,7 +4008,10 @@
       </c>
       <c r="M51" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-2.1.1, GHO-2.1.2, GHO-2.1.3, GHO-2.1.5</t>
+          <t xml:space="preserve">GHO-2.1.1 — Gestion de mensajeria a traves de Visito
+GHO-2.1.2 — Revision y respuesta de correos corporativos
+GHO-2.1.3 — Atencion de canales telefonicos
+GHO-2.1.5 — Informar al personal de recepcion sobre caracteristicas de cada reserva</t>
         </is>
       </c>
       <c r="N51" t="inlineStr" s="2">
@@ -3816,7 +4083,7 @@
       </c>
       <c r="M52" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-2.3.2</t>
+          <t xml:space="preserve">GHO-2.3.2 — Resolucion de conflictos</t>
         </is>
       </c>
       <c r="N52" t="inlineStr" s="2">
@@ -3888,7 +4155,7 @@
       </c>
       <c r="M53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-2.4.2</t>
+          <t xml:space="preserve">GHO-2.4.2 — Orientacion a pasantes o personal de nuevo ingreso</t>
         </is>
       </c>
       <c r="N53" t="inlineStr" s="2">
@@ -3960,12 +4227,17 @@
       </c>
       <c r="M54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-3.3</t>
+          <t xml:space="preserve">GHO-3.3 — Coordinacion de reparaciones tecnicas con personal externo</t>
         </is>
       </c>
       <c r="N54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OPE-3.1, OPE-3.2, OPE-3.4, OPE-4.3, OPE-4.5, OPE-4.6</t>
+          <t xml:space="preserve">OPE-3.1 — Recepcion de solicitud de gerencia
+OPE-3.2 — Recepcion de solicitud de ama de llaves u otros departamentos
+OPE-3.4 — Encomiendas de actividades al equipo operativo
+OPE-4.3 — Recepcion de reporte de ama de llaves
+OPE-4.5 — Ejecucion de las actividades solicitadas
+OPE-4.6 — Atencion de solicitudes de emergencia/inmediatas</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4309,11 @@
       </c>
       <c r="N55" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OPE-4.2, OPE-6.1, OPE-6.2, OPE-6.3, OPE-6.4</t>
+          <t xml:space="preserve">OPE-4.2 — Planificacion de actividades de electricidad
+OPE-6.1 — Verificacion del pozo de agua
+OPE-6.2 — Mantenimiento del pozo
+OPE-6.3 — Verificacion de bombas sumergibles de aguas negras
+OPE-6.4 — Mantenimiento de las bombas sumergibles de aguas negras</t>
         </is>
       </c>
     </row>
@@ -4109,7 +4385,11 @@
       </c>
       <c r="N56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OPE-5.1, OPE-5.3, OPE-5.4, OPE-5.5, OPE-5.6</t>
+          <t xml:space="preserve">OPE-5.1 — Recepcion de solicitud de llenado de tanque de agua
+OPE-5.3 — Recepcion de solicitud de llenado de tanque de gasoil
+OPE-5.4 — Llenado de tanque de gasoil
+OPE-5.5 — Recepcion de solicitud de llenado de tanque de gas
+OPE-5.6 — Llenado de tanque de gas</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4411,7 @@
       </c>
       <c r="D57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COM-Alm-1.12</t>
+          <t xml:space="preserve">COM-Alm-1.12 — Mantenimiento de limpieza del almacen</t>
         </is>
       </c>
       <c r="E57" t="inlineStr" s="2">
@@ -4146,17 +4426,41 @@
       </c>
       <c r="G57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CAJ-1.0, CAJ-1.1, CAJ-1.2, CAJ-1.17, CAJ-4.9, CAJ-4.10</t>
+          <t xml:space="preserve">CAJ-1.0 — Verificacion de lista de huespedes (dia anterior)
+CAJ-1.1 — Encendido de cornetas
+CAJ-1.2 — Encendido de PC, verificacion de Internet e impresora
+CAJ-1.17 — Limpieza de area de caja
+CAJ-4.9 — Limpieza de area (turno tarde)
+CAJ-4.10 — Alimentar a las guacamayas</t>
         </is>
       </c>
       <c r="H57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">BAR-1.1, BAR-1.2, BAR-1.3, BAR-1.4, BAR-1.11, BAR-2.1, BAR-2.3, BAR-2.9, BAR-3.1, BAR-3.2, BAR-3.3, BAR-3.10</t>
+          <t xml:space="preserve">BAR-1.1 — Recepcion de lista de huespedes desde grupo de WhatsApp
+BAR-1.2 — Mise en place de productos y materiales para la produccion
+BAR-1.3 — Verificacion de salon de restaurante
+BAR-1.4 — Limpieza de area de restaurante (apertura, bajo demanda)
+BAR-1.11 — Limpieza de area (cierre de desayuno)
+BAR-2.1 — Limpieza de area de restaurante (periodo de organizacion)
+BAR-2.3 — Prevencion de cualquier pedido de huespedes
+BAR-2.9 — Limpieza de area (cierre de organizacion)
+BAR-3.1 — Mise en place de productos y materiales (turno tarde)
+BAR-3.2 — Verificacion de salon de restaurante (turno tarde)
+BAR-3.3 — Limpieza de area de restaurante (turno tarde, bajo demanda)
+BAR-3.10 — Limpieza de area (cierre de cena)</t>
         </is>
       </c>
       <c r="I57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">COC-1.1, COC-1.4, COC-1.5, COC-2.1, COC-5.3, COC-6.1, COC-6.2, COC-6.3, COC-7.5</t>
+          <t xml:space="preserve">COC-1.1 — Recepcion de lista de desayunos
+COC-1.4 — Desayunos del personal
+COC-1.5 — Desayunos de huespedes
+COC-2.1 — Almuerzos de personal
+COC-5.3 — Cena de personal
+COC-6.1 — Limpieza general del turno de la manana
+COC-6.2 — Limpieza general del turno de la tarde/noche
+COC-6.3 — Solicitud de apoyo a Mantenimiento para casos especiales
+COC-7.5 — Limpieza de area de carniceria</t>
         </is>
       </c>
       <c r="J57" t="inlineStr" s="2">
@@ -4181,7 +4485,15 @@
       </c>
       <c r="N57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OPE-1.1, OPE-1.2, OPE-1.3, OPE-1.4, OPE-2.1, OPE-2.2, OPE-2.3, OPE-4.1, OPE-4.7</t>
+          <t xml:space="preserve">OPE-1.1 — Medicion de cloro y pH
+OPE-1.2 — Aspiracion y retrolavado de piscina
+OPE-1.3 — Activacion de bombas de piscina
+OPE-1.4 — Mantenimiento nocturno de piscina (vertido de cloro)
+OPE-2.1 — Limpieza de areas verdes
+OPE-2.2 — Recoleccion de potes de residuos
+OPE-2.3 — Podar matas
+OPE-4.1 — Apagar luces de areas externas
+OPE-4.7 — Encendido de luces externas</t>
         </is>
       </c>
     </row>
@@ -4233,7 +4545,7 @@
       </c>
       <c r="J58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.4.2</t>
+          <t xml:space="preserve">CCS-4.4.2 — Envio mensual de reporte y pago a Venetur</t>
         </is>
       </c>
       <c r="K58" t="inlineStr" s="2">
@@ -4243,7 +4555,12 @@
       </c>
       <c r="L58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-9.1, AFL-9.2, AFL-9.3, AFL-9.4, AFL-9.5, AFL-9.6</t>
+          <t xml:space="preserve">AFL-9.1 — Exportacion del informe de Ganancias y Perdidas desde Odoo
+AFL-9.2 — Verificacion y clasificacion de los ingresos operativos del dia
+AFL-9.3 — Exportacion del informe de hospedados desde Cloudbeds
+AFL-9.4 — Consolidacion de datos en el archivo Excel para Venetur
+AFL-9.5 — Envio del reporte diario a Venetur
+AFL-9.6 — Envio del reporte de ocupacion a INATUR</t>
         </is>
       </c>
       <c r="M58" t="inlineStr" s="2">
@@ -4285,7 +4602,8 @@
       </c>
       <c r="F59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CTR-6.1, CTR-6.2</t>
+          <t xml:space="preserve">CTR-6.1 — Administracion de usuarios de cuentas bancarias corporativas
+CTR-6.2 — Ejecucion de pagos en plataformas bancarias</t>
         </is>
       </c>
       <c r="G59" t="inlineStr" s="2">
@@ -4305,7 +4623,8 @@
       </c>
       <c r="J59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.1.5, CCS-4.1.6</t>
+          <t xml:space="preserve">CCS-4.1.5 — Apertura de cuentas juridicas
+CCS-4.1.6 — Apertura de cuentas nominas</t>
         </is>
       </c>
       <c r="K59" t="inlineStr" s="2">
@@ -4377,7 +4696,8 @@
       </c>
       <c r="J60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.4.10, CCS-4.1.4</t>
+          <t xml:space="preserve">CCS-4.4.10 — Supervision y conciliacion de ventas ejecutadas por Cashea
+CCS-4.1.4 — Seguimiento y actualizacion de puntos de venta del hotel</t>
         </is>
       </c>
       <c r="K60" t="inlineStr" s="2">
@@ -4449,7 +4769,8 @@
       </c>
       <c r="J61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.6.1, CCS-4.6.2</t>
+          <t xml:space="preserve">CCS-4.6.1 — Actualizacion de inventario intercompany Eracon Salud - SERAC
+CCS-4.6.2 — Actualizacion de inventario intercompany Eracon Alimentos - SERAC</t>
         </is>
       </c>
       <c r="K61" t="inlineStr" s="2">
@@ -4501,7 +4822,12 @@
       </c>
       <c r="F62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CTR-1.1, CTR-1.4, CTR-2.1, CTR-2.2, CTR-2.3, CTR-4.1</t>
+          <t xml:space="preserve">CTR-1.1 — Supervision general de ejecucion de procesos por departamento
+CTR-1.4 — Elaboracion de informe de resultados para gerencia
+CTR-2.1 — Elaboracion del plan de trabajo del departamento de Contraloria
+CTR-2.2 — Identificacion de riesgos y definicion del ambiente de control
+CTR-2.3 — Ejecucion de entrevistas/cuestionarios periodicos a departamentos
+CTR-4.1 — Asesoria estrategica a administracion y talento humano</t>
         </is>
       </c>
       <c r="G62" t="inlineStr" s="2">
@@ -4521,22 +4847,27 @@
       </c>
       <c r="J62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CCS-4.4.1</t>
+          <t xml:space="preserve">CCS-4.4.1 — Seguimiento de gestiones y reportes internos</t>
         </is>
       </c>
       <c r="K62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-1.15, AFJ-1.16, AFJ-1.17, AFJ-8.3</t>
+          <t xml:space="preserve">AFJ-1.15 — Reportar novedades de facturas/pedidos que ameriten correccion
+AFJ-1.16 — Asignacion de actividades en Odoo por informacion o error
+AFJ-1.17 — Seguimiento y cierre de facturas/pedidos con error reportados
+AFJ-8.3 — Informar sobre eventualidades por los distintos medios</t>
         </is>
       </c>
       <c r="L62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-18.1</t>
+          <t xml:space="preserve">AFL-18.1 — Diseno y mantenimiento de formatos operativos</t>
         </is>
       </c>
       <c r="M62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GHO-3.6, GHO-4.4, GHO-5.2</t>
+          <t xml:space="preserve">GHO-3.6 — Chequeo y supervision del personal de A&amp;B
+GHO-4.4 — Supervision del personal de ama de llaves
+GHO-5.2 — Supervision del area de lavanderia en general</t>
         </is>
       </c>
       <c r="N62" t="inlineStr" s="2">
@@ -4603,7 +4934,10 @@
       </c>
       <c r="L63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFL-13.3, AFL-13.4, AFL-13.7, AFL-13.8</t>
+          <t xml:space="preserve">AFL-13.3 — Configuracion de metodos de pago en Cloudbeds
+AFL-13.4 — Creacion de usuarios en Cloudbeds
+AFL-13.7 — Creacion de usuarios en Poster
+AFL-13.8 — Creacion de clientes en Poster</t>
         </is>
       </c>
       <c r="M63" t="inlineStr" s="2">
@@ -4670,7 +5004,8 @@
       </c>
       <c r="K64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AFJ-7.4, AFJ-8.2</t>
+          <t xml:space="preserve">AFJ-7.4 — Atencion y asesoramiento al personal y terceros en procesos
+AFJ-8.2 — Operaciones de soporte administrativo (copias, sello, POS, equipos)</t>
         </is>
       </c>
       <c r="L64" t="inlineStr" s="2">
@@ -4697,16 +5032,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="50" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="38" customWidth="1"/>
-    <col min="8" max="8" width="55" customWidth="1"/>
-    <col min="9" max="9" width="50" customWidth="1"/>
-    <col min="10" max="10" width="45" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="55" customWidth="1"/>
+    <col min="8" max="8" width="45" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4717,7 +5049,7 @@
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Tipo</t>
+          <t xml:space="preserve">Clasificacion</t>
         </is>
       </c>
       <c r="C1" t="inlineStr" s="1">
@@ -4732,7 +5064,7 @@
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Descripcion (el que, no el como)</t>
+          <t xml:space="preserve">Propuesta de solucion</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
@@ -4742,27 +5074,12 @@
       </c>
       <c r="G1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Anclas (Odoo / L10N / DEV)</t>
+          <t xml:space="preserve">Validacion vs doc oficial Odoo 19</t>
         </is>
       </c>
       <c r="H1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Hallazgos RX que resuelve</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Validacion vs doc oficial Odoo 19</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr" s="1">
-        <is>
           <t xml:space="preserve">Doc oficial</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Aliado experto sugerido</t>
         </is>
       </c>
     </row>
@@ -4789,7 +5106,7 @@
       </c>
       <c r="E2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Unificar el alta del proveedor en un unico contacto-proveedor con su RIF, datos bancarios conformes y porcentaje de retencion calificado, eliminando los registros temporales con cuenta personal.</t>
+          <t xml:space="preserve">Implementacion nativa del maestro de proveedores de Odoo (contacto-proveedor unico con RIF, datos bancarios y porcentaje de retencion calificado) que centraliza el alta en un solo registro conforme y elimina los proveedores con cuenta personal creados de forma dispersa en compras y administracion.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="2">
@@ -4799,26 +5116,10 @@
       </c>
       <c r="G2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/purchase/vendor-bills] [L10N:l10n-ve/retenciones]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[COM] Proveedores juridicos se registran con cuentas personales y se aceptan pagos moviles sin cuenta completa, situacion que el AS-IS marca como no conforme al criterio de la empresa y que Contraloria exige corregir; complica ademas las conciliaciones de Administracion.
-[CCS] Al crear un proveedor se valida el porcentaje de retencion calificado en el portal del SENIAT antes de habilitarlo para procesar facturas.</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4847,7 +5148,7 @@
       </c>
       <c r="E3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mantener un maestro unico de productos con categorias que definan las cuentas contables por defecto y variantes por atributos, sustituyendo la asignacion por criterio del equipo y la actualizacion en paralelo en varios sistemas.</t>
+          <t xml:space="preserve">Uso del maestro de productos nativo con categorias que predeterminan el tratamiento contable y variantes por atributos, de modo que el producto se da de alta una sola vez como fuente unica; sustituye la clasificacion por criterio del equipo y elimina la captura paralela del mismo producto en varios sistemas.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="2">
@@ -4857,27 +5158,10 @@
       </c>
       <c r="G3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/accounting/chart-of-accounts] [ODOO:19.0/accounting/taxes]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[CCS] Las categorias de productos se asignaron segun el mejor criterio del equipo y no necesariamente reflejan el tratamiento contable correcto; la revision de cuentas en cada factura corrige manualmente esa configuracion.
-[COM] No existe lista oficial aprobada por Administracion y Contabilidad sobre que productos son almacenables o consumibles; el criterio depende de interpretaciones por area.
-[AFL] Los productos se crean y los precios se actualizan por separado en Odoo, Cloudbeds y Poster, lo que permite discrepancias entre el precio cobrado y el registrado.</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4906,7 +5190,7 @@
       </c>
       <c r="E4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Centralizar el abastecimiento externo en solicitudes de cotizacion a multiples proveedores y ordenes de compra, con acuerdos marco para proveedores recurrentes, en lugar de transcribir compras por indicacion directa sin comparacion de precios.</t>
+          <t xml:space="preserve">Configuracion del flujo de compras nativo (solicitudes de cotizacion a varios proveedores, comparacion y orden de compra, con acuerdos marco para recurrentes) que centraliza todo el abastecimiento externo en un unico circuito con comparacion de precios y elimina las compras transcritas por indicacion directa sin orden previa.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="2">
@@ -4916,30 +5200,10 @@
       </c>
       <c r="G4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/purchase/purchase-order]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[COM] Solo cerca del 10% de las compras pasa por analisis de precio; el 90% restante se transcribe segun la indicacion de Gerencia General sobre a que proveedor comprar, sin presupuesto comparativo.
-[COM] Las condiciones y precios fijos de proveedores constantes se configuran en Odoo, permitiendo generar pedidos recurrentes de forma rapida sin renegociar cada vez.
-[COC] La solicitud de compra que hoy gestiona el almacen cuando no tiene existencia podria originarse desde reglas de reabastecimiento.
-[OPE] La solicitud de materiales faltantes se canaliza a traves de almacen y no directamente al departamento de compras, lo que el equipo senala como ruta incorrecta que anade demora a las reparaciones.
-[BAR] Cuando Almacen no tiene el producto solicitado se gestiona una solicitud de compra, pero no existe sistema que avise al Capitan hasta que el producto llega fisicamente al mostrador.
-[AFJ] Compras que ocurren sin orden previa obligan a montar un pedido a posteriori para dar cobertura contable, generando pedidos abiertos sin receptor formal y retrabajo.</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4968,7 +5232,7 @@
       </c>
       <c r="E5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Registrar las requisiciones internas de reposicion de los departamentos hacia almacen como solicitudes con flujo de aprobacion, sustituyendo el conteo en papel, la lista por WhatsApp y la firma fisica de Gerencia.</t>
+          <t xml:space="preserve">Implementacion de la requisicion interna nativa con flujo de aprobacion en el sistema, que reemplaza el conteo en papel, la lista por WhatsApp y la firma fisica de Gerencia por una solicitud digital trazable y aprobada en linea, eliminando la circulacion de formatos entre areas.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="2">
@@ -4978,30 +5242,10 @@
       </c>
       <c r="G5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/purchase/purchase-order]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[COM] El conteo semanal de viveres, la lista de reposicion y la aprobacion de Gerencia se llevan en papel y se comunican por WhatsApp, sin registro en Odoo del flujo de requisicion-aprobacion.
-[CAJ] El formato manual se anula y rehace completo ante tachaduras, enmiendas o corrector, y circula fisicamente para recabar firma de autorizacion, generando traslados y reprocesos.
-[COC] La solicitud de insumos depende de un formato fisico numerado que debe circular para recabar la firma de Gerencia de Operaciones; si el autorizador no esta presente, la firma queda pendiente y se retrasa la salida de insumos.
-[BAR] La requisicion se llena en papel, circula para recabar la firma de autorizacion de Gerencia de Operaciones y luego se presenta en Almacen para la firma de entrega; un formato fisico que viaja entre areas puede traspapelarse.
-[GHO] A&amp;B, Ama de Llaves y Lavanderia entregan requisiciones en papel que se firman a criterio visual; cocina hace multiples pedidos por semana y lavanderia no lleva control de consumo por ciclo.
-[OPE] La solicitud de insumos a almacen y la entrega de herramientas desde el taller se manejan con formatos fisicos o de forma directa, sin registro.</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5030,7 +5274,7 @@
       </c>
       <c r="E6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ejecutar la recepcion de mercancia como albaran de entrada validado contra la orden de compra y el documento del proveedor antes de confirmar, dando entrada al stock y habilitando la facturacion solo sobre el pedido corregido.</t>
+          <t xml:space="preserve">Uso del albaran de entrada nativo del modulo de inventario, validado contra la orden de compra y el documento del proveedor antes de confirmar, que da entrada al stock y habilita la facturacion solo sobre el pedido conciliado; elimina la desvinculacion entre factura y mercancia y el registro tardio de recepciones.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="2">
@@ -5040,29 +5284,10 @@
       </c>
       <c r="G6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/inventory/delivery-picking] [ODOO:19.0/purchase/vendor-bills]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[COM] El almacen compara la mercancia fisica contra el pedido en Odoo y contra el documento del proveedor, corrige el pedido en Odoo antes de confirmar la recepcion y solo entonces Administracion factura.
-[COC] La recepcion de agua, gas y mercancia que hoy ejecuta Gerencia podria asignarse al area con acceso al sistema mediante el registro de recepciones.
-[AFJ] La norma de que todo pedido pase primero por Almacen con firmas, sellos y documento de entrega corrigio el extravio de documentos y la desvinculacion factura-mercancia.
-[AFL] La recepcion de pedidos y las expediciones entre almacen general y administracion ya se gestionan en Odoo y se sostienen sobre el modulo de inventario, hoy con datos en depuracion.
-[GHO] El agua, el gas y los servicios de reparacion se reciben en Odoo cuando el rol gerencial tiene tiempo; a veces se entera dias despues por factura, retrasando el registro y el pago.</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5091,7 +5316,7 @@
       </c>
       <c r="E7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Modelar el despacho a departamentos internos y la entrega de herramientas como transferencias internas de inventario entre ubicaciones, en lugar del formato fisico que se rehace por errores.</t>
+          <t xml:space="preserve">Uso de las transferencias internas nativas entre ubicaciones para el despacho a departamentos y la entrega de herramientas, que deja respaldo digital de cada salida contra requisicion y elimina el formato fisico que viaja entre areas y se rehace por errores.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="2">
@@ -5101,28 +5326,10 @@
       </c>
       <c r="G7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/inventory/warehouses-locations] [ODOO:19.0/inventory/delivery-picking]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[COM] La salida de mercancia a los departamentos exige requisicion por escrito y se registra como salida de inventario en Odoo, dando respaldo documental al movimiento.
-[CAJ] El movimiento entre sub-almacen de caja y almacen general puede modelarse como transferencia interna con autorizacion, en lugar de formato fisico que se rehace por errores.
-[BAR] El flujo de requisicion fisica con firmas podria manejarse como una solicitud interna de reabastecimiento entre ubicaciones, con su autorizacion registrada, eliminando el traslado del papel entre areas.
-[OPE] La solicitud de insumos a almacen y la salida de material podrian gestionarse como requisiciones y movimientos de inventario, evitando que el operador descubra el faltante en sitio.</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5151,7 +5358,7 @@
       </c>
       <c r="E8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Configurar ubicaciones internas dentro del almacen reflejando el esquema fisico por tipo de producto, en lugar de operar un almacen general unico sin ubicaciones.</t>
+          <t xml:space="preserve">Configuracion de ubicaciones internas dentro del almacen que reflejan el esquema fisico por tipo de producto, dando al sistema la estructura de la que hoy carece al operar con un unico almacen general sin ubicaciones.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="2">
@@ -5161,25 +5368,10 @@
       </c>
       <c r="G8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/inventory/warehouses-locations]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H8" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[COM] La mercancia se ubica fisicamente por tipo de producto, pero Odoo opera con un almacen general unico sin ubicaciones especificas configuradas.</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5208,7 +5400,7 @@
       </c>
       <c r="E9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Llevar el conteo, el inventario ciclico y el ajuste de existencias dentro del modulo de inventario, sustituyendo las hojas fisicas y resolviendo la desalineacion entre el fisico y el sistema mediante recuentos y ajustes registrados.</t>
+          <t xml:space="preserve">Uso del recuento e inventario ciclico nativos del modulo de inventario, que llevan el conteo y el ajuste de existencias al sistema con registro auditable, sustituyen las hojas y libretas fisicas y resuelven la desalineacion entre el stock fisico y el del sistema.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="2">
@@ -5218,31 +5410,10 @@
       </c>
       <c r="G9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/inventory/warehouses-locations] [ODOO:19.0/inventory/lots-serial]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H9" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[COM] Odoo contiene registros desde 2024 y parte de 2025 que no reflejan el inventario fisico real; el almacenista no puede validarlos y realiza el conteo exclusivamente en fisico hasta una toma fisica formal.
-[CTR] Existe un flujo definido y recurrente de seleccion de productos, conteo fisico con el almacenista, verificacion contra sistema y ajuste, con notificacion a gerencia.
-[CAJ] Las verificaciones de nevera, vitrina y almacen de caja (tres veces al dia) se registran en hoja manual sin calculo automatico de reposicion ni respaldo en sistema.
-[COC] La verificacion de stock para cada servicio y el inventario diario del almacen de cocina se hacen por conteo fisico contra un stock ideal anotado a mano, sin sistema.
-[BAR] El inventario de productos, el de barra y el de plateria y manteleria se realizan en libreta o conteo fisico, sin registro digital.
-[AFL] El inventario presenta productos duplicados y referencias incorrectas en depuracion, y la supervision es aleatoria sobre cinco o seis productos sin frecuencia fija.
-[GHO] Las ventas a huespedes registradas en Cloudbeds generan el descuento automatico del stock; el inventario mensual se contrasta fisicamente contra el sistema.</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5271,7 +5442,7 @@
       </c>
       <c r="E10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Definir reglas de reabastecimiento por stock minimo que disparen la reposicion antes del agotamiento, en lugar de la verificacion manual y el calculo mental de disponibilidad.</t>
+          <t xml:space="preserve">Configuracion de las reglas de reabastecimiento nativas por stock minimo, que disparan la reposicion automaticamente antes del agotamiento y eliminan la verificacion manual y el calculo mental de disponibilidad por radio o lista de huespedes.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="2">
@@ -5281,25 +5452,10 @@
       </c>
       <c r="G10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/purchase/purchase-order] [ODOO:19.0/inventory/warehouses-locations]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H10" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[BAR] La confirmacion de que cocina tiene stock suficiente se hace de forma manual y por comunicacion verbal o radio, usando la lista de huespedes como referencia para estimar mentalmente; no hay visibilidad sistematizada del agotamiento de un item.</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5328,7 +5484,7 @@
       </c>
       <c r="E11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Disponer de un punto de venta de restaurante que registre la comanda, asigne mesa o habitacion y enrute el pedido a la estacion de preparacion, sustituyendo la comanda en papel, la doble digitacion y la impresion centralizada en caja.</t>
+          <t xml:space="preserve">Punto de venta de restaurante cuyo nucleo es nativo (comanda, mesa/habitacion y ruteo a la estacion de preparacion) y que elimina la comanda en papel, la doble digitacion y la impresion centralizada en caja; la emision del documento fiscal venezolano requiere desarrollo/integracion de localizacion fiscal sobre ese nucleo.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="2">
@@ -5338,29 +5494,12 @@
       </c>
       <c r="G11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[DEV:pos-restaurante-fiscal-ve]</t>
+          <t xml:space="preserve">POS restaurante (mesas, ruteo a cocina) existe nativo, pero la VENTA emite documento fiscal: El nucleo POS de Odoo es nativo, pero la emision fiscal venezolana (maquina/impresora fiscal homologada, IGTF en ticket, correlativos y formatos fiscales) NO es nativa; requiere desarrollo/integracion de localizacion fiscal VE.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[CAJ] Caja imprime todas las comandas de cocina y barra porque la impresora de cocina esta fuera de servicio; el flujo directo tablet-a-cocina existia antes y dejo de operar, anadiendo carga e intermediacion a caja.
-[BAR] El mesonero anota el pedido a mano y lo traslada fisicamente a Caja, donde recien se digita en Poster; la tablet existe pero no se usa por limitaciones de red, y la impresora de cocina esta fuera de servicio.
-[COC] Almuerzo, snacks y cena dependen de comanderos fisicos que el mesero traslada caminando a cocina; no hay medicion de tiempos pedido-despacho y los tickets pueden mojarse o perderse.</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">POS restaurante (mesas, ruteo a cocina) existe nativo, pero la VENTA emite documento fiscal: El nucleo POS de Odoo es nativo, pero la emision fiscal venezolana (maquina/impresora fiscal homologada, IGTF en ticket, correlativos y formatos fiscales) NO es nativa; requiere desarrollo/integracion de localizacion fiscal VE.</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/sales/point_of_sale/restaurant.html (nucleo no-fiscal)</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -5387,7 +5526,7 @@
       </c>
       <c r="E12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Cerrar el turno de A&amp;B con arqueo de sesion y entrega de guardia en el punto de venta, sustituyendo el cuaderno de novedades y los traspasos informales.</t>
+          <t xml:space="preserve">Uso del cierre de sesion con arqueo nativo del punto de venta, que formaliza la entrega de guardia y la diferencia de efectivo en un acta del sistema y sustituye el cuaderno de novedades, la libreta de faltantes y los traspasos por WhatsApp.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr" s="2">
@@ -5397,28 +5536,12 @@
       </c>
       <c r="G12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/pos/use#close-register]</t>
+          <t xml:space="preserve">Cierre de sesion con arqueo y diferencia de efectivo nativo.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[CAJ] El traspaso de turno y la verificacion de fondo de caja que hoy se anotan en cuaderno de novedades corresponden al cierre de sesion y arqueo nativo del POS.
-[BAR] La entrega de guardia se sustenta en anotaciones informales en la Libreta de Faltantes, el libro de novedades fisico y mensajes de WhatsApp; no existe un acta formal de entrega.</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Cierre de sesion con arqueo y diferencia de efectivo nativo.</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/sales/point_of_sale/use.html</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -5445,7 +5568,7 @@
       </c>
       <c r="E13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Cargar el consumo del huesped desde el punto de venta de A&amp;B al folio de la habitacion para cobro al check-out, sustituyendo el envio Poster-Clover y el control manual de check-outs para no perder cargos.</t>
+          <t xml:space="preserve">Desarrollo/integracion que traslada el consumo del punto de venta de A&amp;B al folio de la habitacion para su cobro unico al check-out, centralizando el cargo en la cuenta del huesped y eliminando el envio Poster-Clover, el control manual de check-outs y los pagos a cuentas personales de mesoneros que hoy generan devoluciones.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr" s="2">
@@ -5455,29 +5578,12 @@
       </c>
       <c r="G13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[DEV:room-charge-folio]</t>
+          <t xml:space="preserve">Cargo de consumo POS al folio de habitacion requiere PMS de terceros o desarrollo.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[CAJ] El envio del consumo de Poster a Clover para cargar a la habitacion apunta a la capacidad de facturar/diferir el cargo a un cliente o folio en el POS.
-[CAJ] Si recepcion no avisa el check-out a tiempo o el envio digital a Clover falla, una comanda puede quedar sin trasladar y el huesped sale sin que se cargue su consumo.
-[GHO] El servicio se cobra exclusivamente por pago movil a la cuenta de los mesoneros; cuando el huesped paga por PDV, se generan dos pagos y una devolucion gestionada con Administracion.</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Cargo de consumo POS al folio de habitacion requiere PMS de terceros o desarrollo.</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">(sin PMS oficial)</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -5504,7 +5610,7 @@
       </c>
       <c r="E14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Relacionar cada plato con sus insumos mediante recetas/escandallos que descuenten la materia prima al producir, sustituyendo el calculo manual de raciones del mise en place.</t>
+          <t xml:space="preserve">Uso de las listas de materiales (escandallos) nativas que relacionan cada plato con sus insumos y descuentan la materia prima al producir o vender, dando una base unica de raciones del mise en place y sustituyendo el calculo manual contra un stock ideal anotado a mano.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr" s="2">
@@ -5514,27 +5620,12 @@
       </c>
       <c r="G14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/mrp/bom-configuration]</t>
+          <t xml:space="preserve">BOM/escandallos con consumo de componentes nativo (descuento por venta POS para A&amp;B).</t>
         </is>
       </c>
       <c r="H14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[COC] El calculo de raciones por ingrediente en el mise en place y el descuento de insumos al producir podria apoyarse en listas de materiales/recetas que relacionan plato e insumos.</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">BOM/escandallos con consumo de componentes nativo (descuento por venta POS para A&amp;B).</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/inventory_and_mrp/manufacturing/basic_setup/bill_configuration.html</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -5561,7 +5652,7 @@
       </c>
       <c r="E15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Registrar la produccion de proteinas de carniceria y sus descartes como movimientos de ajuste/desecho de inventario, dando seguimiento historico de merma sobre el insumo de mayor valor.</t>
+          <t xml:space="preserve">Uso de los movimientos de desecho y ajuste nativos del inventario para registrar la produccion de carniceria y sus descartes, que consolida un historico estructurado de merma sobre el insumo de mayor valor y sustituye las hojas de produccion en papel y el control manual contra el peso inicial.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr" s="2">
@@ -5571,25 +5662,10 @@
       </c>
       <c r="G15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/inventory/lots-serial]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H15" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[COC] El conteo de proteinas procesadas se registra a mano en hojas de produccion y la merma se controla por revision manual contra el peso inicial; las diferencias se escalan a Gerencia, pero no hay registro estructurado que permita seguimiento historico de mermas.</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5618,7 +5694,7 @@
       </c>
       <c r="E16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Controlar el prestamo de cavas al huesped mediante numeros de serie y un registro de salida y devolucion, en lugar del listado manual sin identificacion univoca.</t>
+          <t xml:space="preserve">Uso del seguimiento por numero de serie nativo del inventario para identificar cada cava de forma univoca y registrar su salida y devolucion, dando trazabilidad al prestamo y eliminando el listado manual de caja que no distingue una cava de otra.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr" s="2">
@@ -5628,25 +5704,10 @@
       </c>
       <c r="G16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/inventory/lots-serial]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H16" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[CAJ] El prestamo de cavas se gestiona en un listado manual exclusivo de caja, sin numero grabado por cava ni registro digital; el AS-IS senala que no se lleva orden ni conteo y que el huesped podria devolver una distinta sin que se note.</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5675,7 +5736,7 @@
       </c>
       <c r="E17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Registrar el efectivo de los cierres de turno de cada punto de venta en los diarios de caja y conciliar el efectivo entregado contra los reportes del sistema y los comprobantes, formalizando la doble revision.</t>
+          <t xml:space="preserve">Uso de los diarios de efectivo nativos para registrar el cierre de cada punto de venta y conciliar el efectivo entregado contra los reportes del sistema, los comprobantes electronicos y los reportes de punto de venta bancario, dejando la doble revision como un control formal en linea y eliminando la consolidacion en Excel publicada en Teams.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr" s="2">
@@ -5685,26 +5746,10 @@
       </c>
       <c r="G17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/accounting/customer-invoice] [ISO:9001:2015 §8.5.1]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H17" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[AFL] Cada cierre de turno se valida primero por el punto de venta (recepcion o A&amp;B) y luego por Administracion, cruzando el sistema (Cloudbeds/Poster) contra el efectivo fisico, los reportes de punto de venta bancario y los comprobantes electronicos antes de aceptar la entrega.
-[GHO] El cierre de turno se consolida en Excel y se publica en Teams; el control de redobles depende de una agenda fisica.</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5733,7 +5778,7 @@
       </c>
       <c r="E18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Registrar el cobro del huesped como recibo de cobro vinculado a su factura una vez confirmado el ingreso en banco, eliminando el triple registro manual (Cloudbeds, Odoo, Teams) del mismo pago.</t>
+          <t xml:space="preserve">Uso del recibo de cobro nativo vinculado a la factura del huesped, registrado una sola vez al confirmar el ingreso en banco, que centraliza el cobro en el sistema contable y elimina el triple registro manual del mismo pago entre Cloudbeds, Odoo y la carpeta de Teams.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr" s="2">
@@ -5743,27 +5788,10 @@
       </c>
       <c r="G18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/accounting/customer-invoice]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H18" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[GHO] Cada pago se carga en Cloudbeds, luego en Odoo (recibo de cliente) y luego se copia/pega en una carpeta de Microsoft Teams con el comprobante adjunto. La misma transaccion se reescribe en tres entornos sin integracion.
-[AFL] Ningun pago movil o transferencia se da por valido hasta confirmarse su ingreso real en el portal del banco, dato que se devuelve sobre el propio comprobante.
-[AFL] Como la caja de A&amp;B no tiene usuario de Odoo, Administracion registra manualmente cada recibo de cobro (uno por pago) y la factura de consumos al cierre, duplicando el trabajo ya capturado en Poster.</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5792,7 +5820,7 @@
       </c>
       <c r="E19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Importar los extractos bancarios y los lotes de POS y conciliarlos contra los recibos y pagos mediante reglas de conciliacion, sustituyendo el cotejo manual de extractos, comisiones y tasas.</t>
+          <t xml:space="preserve">Uso de la conciliacion bancaria nativa con importacion de extractos (y lotes de POS via diarios puente) y reglas de conciliacion, que cruza automaticamente los movimientos de banco contra recibos y pagos y sustituye el cotejo manual de extractos de varios bancos, comisiones, tasas y lotes de Credicard; los estados de cuenta dejan de mantenerse en paralelo en Excel.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr" s="2">
@@ -5802,30 +5830,12 @@
       </c>
       <c r="G19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/finance/accounting/bank/transactions] [ODOO:19.0/finance/accounting/bank/reconciliation]</t>
+          <t xml:space="preserve">Importacion de extractos (CAMT/CSV/OFX/QIF) + reglas de conciliacion nativo; pagos POS via diarios puente.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[CCS] El cotejo manual de extractos, comisiones y EDC podria apoyarse en la conciliacion bancaria de Odoo con reglas de conciliacion.
-[AFJ] La conciliacion pago-extracto es diaria y la ejecutan varios roles; los pagos devueltos no detectados a tiempo generan notas de debito, disputas y retrabajo que toman de dias a semanas.
-[AFL] El cruce manual de extractos descargados de Banesco, Banplus, Bancamiga y Banco Exterior, y de lotes de Credicard, contra los recibos de cobro podria apoyarse en la conciliacion nativa con importacion de extractos bancarios.
-[RRH] La conciliacion se valida en Odoo pero los estados de CxC por trabajador se mantienen manualmente en Excel, generando desfases temporales entre ambos.</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Importacion de extractos (CAMT/CSV/OFX/QIF) + reglas de conciliacion nativo; pagos POS via diarios puente.</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/finance/accounting/bank/reconciliation.html</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -5852,7 +5862,7 @@
       </c>
       <c r="E20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conciliar los recibos de efectivo y de divisas digitales contra extractos de caja y de plataformas, y distinguir el estado de factura pagada de la conciliacion pendiente, sin crear los extractos a mano.</t>
+          <t xml:space="preserve">El nucleo es la conciliacion nativa de diarios de caja y multimoneda, que distingue la factura pagada de la conciliacion pendiente y resuelve la confusion de saldos; la carga de los extractos de caja fisica y de plataformas de divisas (PayPal, Binance, Zelle), hoy creados a mano, requiere desarrollo de integracion para evitar ese registro manual.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="2">
@@ -5862,28 +5872,12 @@
       </c>
       <c r="G20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/finance/accounting/bank/reconciliation] [DEV:integracion-plataformas-divisas]</t>
+          <t xml:space="preserve">Conciliacion caja/multimoneda nativa; integracion con plataformas de divisas digitales = desarrollo.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[AFL] A diferencia del extracto bancario importable, los extractos de la caja fisica y de las plataformas de divisas (PayPal, Binance, Zelle) se crean manualmente en Odoo antes de poder conciliar los recibos de cobro.
-[AFL] Una factura con saldo cero pero sin conciliar permanece en En proceso de pago en lugar de Pagada, generando confusion operativa sobre el estado real del cobro.</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Conciliacion caja/multimoneda nativa; integracion con plataformas de divisas digitales = desarrollo.</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/finance/accounting/bank/reconciliation.html</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -5910,7 +5904,7 @@
       </c>
       <c r="E21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Emitir las facturas de venta de los servicios del hotel con el motor de impuestos y la gestion multimoneda del sistema, discriminando la base imponible del IVA sin Excel externo.</t>
+          <t xml:space="preserve">Uso del motor de impuestos y la gestion multimoneda nativos para emitir las facturas de venta de los servicios del hotel, que calculan y discriminan la base imponible del IVA dentro del sistema y eliminan el Excel auxiliar de tasa promedio y discriminacion de base por factura.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="2">
@@ -5920,26 +5914,10 @@
       </c>
       <c r="G21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/accounting/customer-invoice] [ODOO:19.0/accounting/taxes] [NORMA:LIVA Art. 20, 28-29]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H21" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[AFL] Para cada factura se descarga la cuenta del cliente a un Excel auxiliar donde se calcula la tasa promedio de pagos en distintas fechas y se discrimina la base imponible, porque Odoo recibe la base y no el total con IVA.
-[AFL] Todas las facturas (recepcion, A&amp;B, estacionamiento, Marina, arrendamientos) se emiten como facturas de contingencia y se imprimen en impresora comun por no contar con maquina fiscal integrada.</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5968,7 +5946,7 @@
       </c>
       <c r="E22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sostener tarifas por segmento (agencias, grupos) y reglas de descuento en listas de precio sobre el catalogo unico, reduciendo la consulta caso por caso a presidencia y la desincronizacion del menu.</t>
+          <t xml:space="preserve">Uso de las listas de precio nativas para parametrizar tarifas por segmento (agencias, grupos, eventos) y descuentos sobre el catalogo unico, dejando el precio predefinido en el sistema; elimina la consulta caso por caso a presidencia y la desincronizacion del menu impreso frente al precio cobrado.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr" s="2">
@@ -5978,26 +5956,10 @@
       </c>
       <c r="G22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/sales/pricelists]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H22" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[GHO] Comisiones de agencias, descuentos de grupos/eventos y compensaciones se consultan individualmente con presidencia/gerencia, sin tabla de tarifas o descuentos predefinida; la demora hace perder clientes.
-[AFL] El menu impreso en Canva puede quedar desincronizado de los precios de Poster, obligando a reimprimir y arriesgando cobrar un precio distinto al registrado.</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6026,7 +5988,7 @@
       </c>
       <c r="E23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Gestionar las cuentas por pagar por vencimiento y antiguedad de saldos directamente sobre las facturas de proveedor, e incorporar las obligaciones recurrentes, sustituyendo la plantilla manual de Excel y el reporte diario por WhatsApp.</t>
+          <t xml:space="preserve">Uso del reporte de antiguedad de saldos por pagar nativo, alimentado directamente por las facturas de proveedor y las obligaciones recurrentes registradas (servicios fijos mensuales), que centraliza la planificacion de pagos en el sistema y sustituye la plantilla manual de CxP en Excel actualizada tres veces al dia.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="2">
@@ -6036,28 +5998,10 @@
       </c>
       <c r="G23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/purchase/vendor-bills]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H23" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[AFJ] La relacion de CxP se mantiene manualmente en Excel porque el modulo de Compras contiene pedidos basura que impiden extraer la informacion directa del sistema; la actualizacion se hace tres veces al dia.
-[AFJ] Facturas de proveedores con factura directa y servicios fijos mensuales (CORPOELEC, TELMACA, seguridad) deben cargarse a mano en el Excel o quedan fuera de la planificacion de pagos.
-[CCS] La planificacion de pagos depende de una plantilla manual de cuentas por pagar en Excel para identificar vencimientos y priorizar, manteniendo doble gestion respecto del sistema contable.
-[COM] El estado de los pedidos (cerrados, por facturar, por recibir) se revisa al cierre de cada quincena cruzando los modulos de Compras e Inventario, y se entrega informe al tesorero.</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6086,7 +6030,7 @@
       </c>
       <c r="E24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Registrar la factura de proveedor, ejecutar el pago contra el pedido autorizado y aplicar/conciliar la partida en el sistema, cerrando el ciclo de compra a pago.</t>
+          <t xml:space="preserve">Uso de las facturas de proveedor y los pagos nativos vinculados al pedido autorizado, que cierran el ciclo de compra a pago dentro del sistema (validacion documental, ejecucion del pago y aplicacion/conciliacion de la partida) y dan estado unico al avance de cada pago en lugar del control disperso por tarjeta y por archivo manual.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="2">
@@ -6096,28 +6040,10 @@
       </c>
       <c r="G24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/purchase/vendor-bills]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H24" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[AFJ] La revision documental contra requisitos SENIAT y la verificacion de tasa de cambio antes de registrar funcionan como control de calidad robusto en el primer eslabon.
-[CCS] Todo pago a proveedores se verifica contra un pedido previamente autorizado por la Gerencia General antes de ejecutarse desde la plataforma bancaria.
-[CCS] Las 23 tarjetas se pagan una a una con un archivo manual y la conciliacion se imputa tarjeta por tarjeta; no existe un sistema interno que mida el estado de corte de cada tarjeta.
-[AFL] Todo pago a proveedores o empleados desde la caja principal exige autorizacion previa de la Gerencia General, recibo fisico firmado por el receptor y conciliacion posterior en Odoo por el area responsable.</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6146,7 +6072,7 @@
       </c>
       <c r="E25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Registrar los anticipos a proveedor y aplicarlos a la factura como partidas pendientes del sistema, facilitando la depuracion de los saldos antiguos abiertos.</t>
+          <t xml:space="preserve">Uso de los anticipos y pagos pendientes nativos para registrar el adelanto al proveedor y aplicarlo a su factura dentro del sistema, sustituyendo la carpeta local y los recordatorios manuales y facilitando la depuracion de los saldos de anticipo antiguos que hoy quedan abiertos y distorsionan el balance.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="2">
@@ -6156,25 +6082,10 @@
       </c>
       <c r="G25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/purchase/vendor-bills]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H25" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[AFJ] El control de pagos anticipados se apoya en una carpeta local del computador y en recordatorios; la depuracion de saldos de anticipo 2023-2024 es compleja y voluminosa, y los anticipos antiguos quedan abiertos distorsionando el balance.</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6203,7 +6114,7 @@
       </c>
       <c r="E26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Diferenciar contablemente las deudas y pagos con socios respecto de los proveedores externos y registrar las cuentas por cobrar a socios, evitando que distorsionen el saldo de proveedores.</t>
+          <t xml:space="preserve">Uso de cuentas y partidas contables dedicadas para separar las deudas y cobros con socios de los proveedores externos, que aisla la posicion real de CxP y CxC y elimina la acumulacion de pagos de socios como deuda a proveedor que hoy distorsiona el saldo.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="2">
@@ -6213,25 +6124,10 @@
       </c>
       <c r="G26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/accounting/chart-of-accounts]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H26" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[CCS] Los asientos de facturas pagadas por los socios se acumulan como CxP a proveedor cuando la deuda real es con el socio que efectuo el pago, distorsionando el saldo de proveedores y la posicion real de CxP.</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6260,7 +6156,7 @@
       </c>
       <c r="E27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Procesar las devoluciones por error de costo o cantidad mediante notas de credito y reversiones, en lugar de la deteccion tardia y devolucion manual.</t>
+          <t xml:space="preserve">Uso de las notas de credito y reversiones nativas para procesar los errores de costo o cantidad de la factura de proveedor, dejando el ajuste documentado en el sistema en lugar de la devolucion manual que hoy se detecta tarde y retrasa el pago.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="2">
@@ -6270,25 +6166,10 @@
       </c>
       <c r="G27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/accounting/credit-debit-notes]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H27" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[CCS] Los errores de costo o cantidad se detectan al procesar la factura, 7 a 15 dias despues de que Compras monto el pedido y Almacen lo recepciono, generando devoluciones que retrasan el pago al proveedor.</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6317,7 +6198,7 @@
       </c>
       <c r="E28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Generar los comprobantes y archivos de retencion de IVA e ISLR con la localizacion fiscal venezolana, eliminando la correccion manual de XML y la macro externa, y registrar el seguimiento de reembolsos de retencion.</t>
+          <t xml:space="preserve">Uso de las retenciones de la localizacion fiscal venezolana para calcular y emitir los comprobantes y archivos de retencion de IVA e ISLR del periodo dentro del sistema, eliminando la correccion manual de XML y la macro externa de consolidacion; deja el certificado y el seguimiento de reembolsos de retencion en un unico flujo formal.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="2">
@@ -6327,30 +6208,10 @@
       </c>
       <c r="G28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/accounting/withholding-taxes] [L10N:l10n-ve/retenciones] [NORMA:retencion IVA/ISLR contribuyente especial SENIAT]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H28" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[CCS] La version actual de Odoo genera XML invalido cuando una factura tiene mas de dos impuestos o base imponible alterada, lo que obliga a correccion manual antes de enviar al contador, bajo riesgo de rechazo del SENIAT.
-[CCS] Odoo no genera el XML de retencion sobre nomina; se produce con una macro manual y se fusiona con el XML de compras, proceso enteramente manual de consolidacion.
-[AFJ] La generacion, validacion quincenal y emision del certificado de retencion ya se apoyan en Odoo; la localizacion fiscal venezolana es el marco nativo para sostener este flujo.
-[AFL] El registro de los comprobantes de retencion de contribuyentes especiales corresponde a la funcionalidad de retenciones de la localizacion fiscal venezolana.
-[COM] La recuperacion de retenciones de IVA/ISLR ante proveedores que exigen pago completo se gestiona solo por correo con insistencia manual, sin mecanismo formal de seguimiento.
-[RRH] Elaboracion de archivo XML para declaracion de retenciones ISLR.</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6379,7 +6240,7 @@
       </c>
       <c r="E29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Producir el libro de compras del periodo y soportar el cierre fiscal quincenal desde el diario contable, reduciendo el escaneo, conteo y enumeracion manual de documentos.</t>
+          <t xml:space="preserve">Uso del libro de compras de la localizacion venezolana generado desde el diario contable, que produce el documento integro del periodo para el cierre quincenal del contribuyente especial y reduce el conteo, escaneo y enumeracion manual de facturas que hoy provoca descuadres entre libros.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="2">
@@ -6389,26 +6250,10 @@
       </c>
       <c r="G29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[L10N:l10n-ve/libros-fiscales] [NORMA:contribuyente especial IVA quincenal SENIAT]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H29" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[AFJ] El conteo exacto de facturas escaneadas contra las declaradas y la numeracion del libro de compras solo cuando el periodo esta cerrado garantizan que el libro a declarar sea integro.
-[CTR] Los libros de IVA compras y ventas no cuadran cada mes, generando inconsistencias en los libros fiscales.</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6437,7 +6282,7 @@
       </c>
       <c r="E30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Bloquear las fechas de los periodos contables cerrados para impedir la modificacion retroactiva y emitir los libros legales (diario, mayor, inventario) exigidos por el Codigo de Comercio.</t>
+          <t xml:space="preserve">Uso del bloqueo de fechas y los reportes contables nativos, que cierran los periodos para impedir la modificacion retroactiva (devolviendo confiabilidad a los reportes ya emitidos) y emiten los libros legales de diario, mayor e inventario exigidos por el Codigo de Comercio que hoy no se imprimen.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="2">
@@ -6447,26 +6292,10 @@
       </c>
       <c r="G30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/accounting/chart-of-accounts] [NORMA:Codigo de Comercio Art. 32-34]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H30" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[CTR] Los reportes descargados no son confiables porque periodos anteriores siguen siendo modificados, alterando cifras de reportes ya emitidos e invalidando analisis previos.
-[CTR] Falta incorporar libro diario, libro de inventario y balance; el Codigo de Comercio exige impresion mensual y no se cumple por ausencia de cierres.</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6495,7 +6324,7 @@
       </c>
       <c r="E31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Registrar los aportes parafiscales y municipales de fecha fija (FONACIT, INATUR, Alcaldia, INPARQUES, aseo urbano, VACC) como obligaciones contables con su base y vencimiento, evitando multas por incumplimiento de plazo.</t>
+          <t xml:space="preserve">Registro de los aportes parafiscales y municipales de fecha fija (FONACIT, INATUR, Alcaldia, INPARQUES, aseo urbano, VACC) como obligaciones contables recurrentes con base y vencimiento en el sistema, dando visibilidad de los plazos y evitando las multas por incumplimiento que hoy dependen del seguimiento manual de cada fecha.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="2">
@@ -6505,25 +6334,10 @@
       </c>
       <c r="G31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[NORMA:obligaciones parafiscales y municipales VE] [L10N:l10n-ve/impuestos-municipales]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H31" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[CCS] INPARQUES (dia 5), INATUR (dia 5), Alcaldia Silva (dia 15), VACC (dia 10) y la facturacion intercompany de Eracon Alimentos tienen plazos estrictos cuyo incumplimiento genera multa.</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6552,7 +6366,7 @@
       </c>
       <c r="E32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Soportar el cumplimiento parafiscal laboral y las declaraciones de tributos sobre nomina (ARC/ARI, IPP, ISLR/IGP) con el mecanismo de retenciones de la localizacion venezolana.</t>
+          <t xml:space="preserve">Uso del mecanismo de retenciones de la localizacion venezolana para soportar el cumplimiento parafiscal laboral y las declaraciones de tributos sobre nomina (ARC/ARI, IPP, ISLR/IGP) sobre saldos del propio sistema, reduciendo la dependencia del criterio externo del contador y la consolidacion manual.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="2">
@@ -6562,26 +6376,10 @@
       </c>
       <c r="G32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/accounting/withholding-taxes] [L10N:l10n-ve/retenciones] [NORMA:LOTTT — obligaciones parafiscales del empleador]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H32" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[RRH] El area ejecuta un ciclo definido de revision, validacion, solicitud de compromiso de pago y archivo para IVSS, INCES, FAOV y MPPPST, con documentacion consolidada en la carpeta Oslo.
-[CCS] Los cierres y cuadres no razonables en Odoo obligan a que el contador externo elabore una propuesta de trabajo para declarar ISLR e IGP, dependiendo de un criterio externo en lugar de saldos del sistema.</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6610,7 +6408,7 @@
       </c>
       <c r="E33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Centralizar el archivo digital ordenado por departamento y periodo y la gestion de notificaciones de entes, sustituyendo el archivo reactivo en nube sin estructura y la busqueda de urgencia ante fiscalizaciones.</t>
+          <t xml:space="preserve">Uso del modulo de gestion documental (Enterprise) con espacios por departamento y periodo, etiquetas, permisos y alias de correo, que centraliza el archivo digital ordenado y el flujo de notificaciones de entes, sustituyendo el archivo reactivo en nube sin estructura y la busqueda de urgencia ante fiscalizaciones.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="2">
@@ -6620,30 +6418,12 @@
       </c>
       <c r="G33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/productivity/documents]</t>
+          <t xml:space="preserve">Documents (Enterprise): workspaces/carpetas, etiquetas, permisos, alias de correo.</t>
         </is>
       </c>
       <c r="H33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[CTR] Desde 2023 la documentacion no se archiva preventivamente; al llegar una fiscalizacion los departamentos buscan y escanean papeles de urgencia, con riesgo de presentar informacion incompleta.
-[RRH] No existe registro interno estandarizado ni flujo con responsables y plazos para atender notificaciones de inspecciones gubernamentales.
-[AFJ] La factura original solo llega despues del pago y los documentos se acumulan hasta el envio trimestral de la valija a Caracas; el incumplimiento en el archivo y disponibilidad en la nube es sancionable.
-[CCS] Existe un acumulado de facturas fiscales de compra y venta pendiente de archivar y ordenar, ejecutado de forma esporadica y con apoyo variable.</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Documents (Enterprise): workspaces/carpetas, etiquetas, permisos, alias de correo.</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/productivity/documents.html</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -6670,7 +6450,7 @@
       </c>
       <c r="E34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Marcar el seguimiento de la recepcion de la guia SUNAGRO SICA dentro del plazo del portal; capacidad sectorial sin via nativa ni de localizacion disponible.</t>
+          <t xml:space="preserve">Capacidad sectorial sin via nativa ni de localizacion: el seguimiento de la guia SUNAGRO SICA dentro del plazo del portal requiere desarrollo de integracion con el portal estatal para dar alerta del vencimiento y evitar la multa, ya que Odoo no la cubre de forma estandar.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="2">
@@ -6680,27 +6460,12 @@
       </c>
       <c r="G34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[DEV:integracion-SUNAGRO-SICA]</t>
+          <t xml:space="preserve">Seguimiento guia SUNAGRO SICA: portal estatal VE, sin via nativa.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[AFJ] La guia tiene fecha de vencimiento para su recepcion en el portal; el incumplimiento genera multa y medidas disciplinarias de gerencia.</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Seguimiento guia SUNAGRO SICA: portal estatal VE, sin via nativa.</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">(portal gubernamental VE)</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -6727,7 +6492,7 @@
       </c>
       <c r="E35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Calcular y procesar la nomina, las horas extras, los bonos, los descuentos y las liquidaciones con estructuras y reglas salariales del modulo de nomina, sustituyendo las hojas de Excel paralelas.</t>
+          <t xml:space="preserve">El nucleo es el motor de nomina nativo (Enterprise) con estructuras y reglas salariales que procesa conceptos, horas extras, bonos, descuentos y liquidaciones y elimina las hojas de Excel paralelas con transcripcion manual; las reglas venezolanas (LOTTT, IVSS, FAOV, INCES) no tienen localizacion oficial y requieren configuracion/desarrollo o modulo de tercero.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="2">
@@ -6737,27 +6502,12 @@
       </c>
       <c r="G35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/hr/payroll] [DEV:l10n-ve-payroll]</t>
+          <t xml:space="preserve">Motor de nomina nativo (Enterprise) pero NO hay localizacion VE oficial; reglas LOTTT/IVSS/FAOV/INCES = config/desarrollo o modulo de tercero.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] Todo el procesamiento de pago se realiza en hojas paralelas, con consolidacion, sumatorias y transcripcion manuales sujetas a error y reproceso.</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Motor de nomina nativo (Enterprise) pero NO hay localizacion VE oficial; reglas LOTTT/IVSS/FAOV/INCES = config/desarrollo o modulo de tercero.</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/hr/payroll.html</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -6784,7 +6534,7 @@
       </c>
       <c r="E36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Generar el archivo de pago bancario de la nomina y las horas extras desde el sistema, sustituyendo la elaboracion manual del TXT y las transferencias individuales.</t>
+          <t xml:space="preserve">El pago por lote es nativo, pero usa el formato SEPA: generar el archivo TXT del banco venezolano desde la nomina requiere desarrollo del formato de pais, con lo que el archivo de pago de nomina y horas extras sale del sistema y sustituye la elaboracion manual del TXT y las transferencias una a una.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="2">
@@ -6794,27 +6544,12 @@
       </c>
       <c r="G36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/hr/payroll] [DEV:archivo-pago-banco-ve]</t>
+          <t xml:space="preserve">Pago batch nativo es SEPA; archivo TXT por banco venezolano = desarrollo de formato.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] Elaboracion de archivo masivo (TXT) para pago de horas extras y nomina; transferencias individuales a colaboradores con cuentas de otros bancos.</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Pago batch nativo es SEPA; archivo TXT por banco venezolano = desarrollo de formato.</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/hr/payroll.html</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -6841,7 +6576,7 @@
       </c>
       <c r="E37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Registrar la asistencia, los retardos y las horas extras digitalmente para que alimenten el calculo de nomina, sustituyendo Tango Uno, el listado manual y los formatos fisicos.</t>
+          <t xml:space="preserve">Uso del modulo de asistencias nativo para capturar fichaje, retardos con tolerancia y horas extras que alimentan directamente la nomina, unificando en el sistema lo que hoy se reparte entre Tango Uno, un listado manual, Excel y formatos fisicos y eliminando los descuentos incorrectos por coberturas no notificadas.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="2">
@@ -6851,28 +6586,12 @@
       </c>
       <c r="G37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/hr/attendances]</t>
+          <t xml:space="preserve">Asistencia, retardos (tolerancia), horas extra que alimentan nomina, nativo.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] La asistencia se lleva entre Tango Uno, un listado manual y Excel; las horas extras circulan en formatos fisicos impresos y distribuidos, con riesgo de descuentos incorrectos por coberturas no notificadas.
-[GHO] El control de redobles depende de una agenda fisica, con riesgo de olvido si no se anota en el momento.</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Asistencia, retardos (tolerancia), horas extra que alimentan nomina, nativo.</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/hr/attendances.html</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -6899,7 +6618,7 @@
       </c>
       <c r="E38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Canalizar la captacion y preseleccion de candidatos en un pipeline unico de reclutamiento con postulaciones y documentacion, sustituyendo la recepcion dispersa de curriculos y la preseleccion sin formato.</t>
+          <t xml:space="preserve">Uso del pipeline de reclutamiento nativo con etapas, postulaciones y documentacion, que canaliza la captacion y preseleccion en un unico flujo comparable y sustituye la recepcion de curriculos por correo, presencial y grupos dispersos y la preseleccion sin formato.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="2">
@@ -6909,28 +6628,12 @@
       </c>
       <c r="G38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/hr/recruitment]</t>
+          <t xml:space="preserve">Pipeline de reclutamiento con etapas, postulaciones y documentacion, nativo.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] La preseleccion se basa en criterio profesional sin formato estructurado; los curriculos llegan por correo, presencial y grupos dispersos, dificultando la comparacion objetiva.
-[GHO] Analisis de perfiles para reclutamiento de recepcion.</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Pipeline de reclutamiento con etapas, postulaciones y documentacion, nativo.</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/hr/recruitment.html</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -6957,7 +6660,7 @@
       </c>
       <c r="E39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Capturar la informacion integral del empleado (salud, carga familiar, estado civil, datos bancarios, foto), el expediente y el organigrama en un registro unico, eliminando la base Excel paralela y la dispersion en multiples repositorios.</t>
+          <t xml:space="preserve">Uso del maestro de empleado nativo (datos personales y bancarios, salud, carga familiar, estado civil, foto, expediente y organigrama) como registro unico, que elimina la base de datos paralela en Excel y la dispersion del expediente entre fisico, OneDrive/SharePoint y Odoo.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="2">
@@ -6967,27 +6670,12 @@
       </c>
       <c r="G39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/hr/employees]</t>
+          <t xml:space="preserve">Maestro de empleado (datos personales, bancarios, dependientes, foto), expediente y organigrama nativo.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] La base de datos detallada vive en Excel (activos/egresados) porque Odoo no captura salud, carga familiar, estado civil ni datos bancarios; coexiste con expedientes fisicos, OneDrive/SharePoint y Odoo.</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Maestro de empleado (datos personales, bancarios, dependientes, foto), expediente y organigrama nativo.</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/hr/employees.html</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7014,7 +6702,7 @@
       </c>
       <c r="E40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Gestionar la incorporacion y el egreso (induccion, contrato, liquidacion, devolucion de activos, baja y revocacion de accesos) como un flujo registrado del empleado, formalizando las aprobaciones hoy verbales.</t>
+          <t xml:space="preserve">El nucleo son los planes de actividades nativos de onboarding/offboarding que registran induccion, contrato, devolucion de activos y baja con sus aprobaciones, formalizando lo que hoy se transmite verbalmente o por WhatsApp; la revocacion de accesos y la liquidacion dependen de pasos no nativos y de Payroll, por lo que parte requiere configuracion/desarrollo.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="2">
@@ -7024,28 +6712,12 @@
       </c>
       <c r="G40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/hr/employees/offboarding] [DEV:revocacion-accesos]</t>
+          <t xml:space="preserve">Onboarding/offboarding via planes de actividades nativo; revocacion de accesos/usuario no es paso nativo; liquidacion depende de Payroll.</t>
         </is>
       </c>
       <c r="H40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] El egreso integra notificacion a departamentos, baja en Odoo y canales, revocacion de accesos por IT y verificacion de devolucion de uniformes y equipos mediante checklist.
-[RRH] La aprobacion final de ingreso por Gerencia General, los cambios de condiciones laborales y varias notificaciones se transmiten verbalmente o por WhatsApp, sin respaldo escrito sistematico.</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Onboarding/offboarding via planes de actividades nativo; revocacion de accesos/usuario no es paso nativo; liquidacion depende de Payroll.</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/hr/employees/offboarding.html</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7072,7 +6744,7 @@
       </c>
       <c r="E41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Atender permisos, reposos, vacaciones, prestamos y dias libres como solicitudes de ausencia con flujo de aprobacion registrado, sustituyendo los recibos manuales y la planificacion en Excel.</t>
+          <t xml:space="preserve">Uso del modulo de ausencias nativo para gestionar permisos, reposos, vacaciones, prestamos y dias libres con aprobacion y acumulacion registradas, sustituyendo los recibos manuales y la planificacion de vacaciones y horarios en Excel.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="2">
@@ -7082,28 +6754,12 @@
       </c>
       <c r="G41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/hr/time_off]</t>
+          <t xml:space="preserve">Permisos, reposos, vacaciones, dias libres con aprobacion y acumulacion, nativo.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] Las solicitudes en recibos manuales y la planificacion de vacaciones en Excel podrian atenderse con solicitudes de ausencia y aprobaciones registradas.
-[GHO] Elaboracion de horarios del departamento y planificacion estrategica de equipos para temporadas altas.</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Permisos, reposos, vacaciones, dias libres con aprobacion y acumulacion, nativo.</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/hr/time_off.html</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7130,7 +6786,7 @@
       </c>
       <c r="E42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ejecutar la evaluacion de desempeno por cargo con indicadores y escala dentro del sistema, conservando el mecanismo formal existente.</t>
+          <t xml:space="preserve">Uso del modulo de evaluacion de desempeno nativo (plantillas con indicadores por cargo, metas y escala), que lleva al sistema el mecanismo formal ya existente y consolida los resultados en el expediente del empleado en lugar de plantillas sueltas.</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="2">
@@ -7140,27 +6796,12 @@
       </c>
       <c r="G42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/hr/appraisals]</t>
+          <t xml:space="preserve">Evaluacion de desempeno con plantillas, metas y escala, nativo.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] Existen plantillas predeterminadas con 20-25 indicadores por cargo y escala 1-5, aplicadas al cierre del periodo de prueba con participacion del coordinador de area.</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Evaluacion de desempeno con plantillas, metas y escala, nativo.</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/hr/appraisals.html</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7187,7 +6828,7 @@
       </c>
       <c r="E43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Registrar la entrega y devolucion de uniformes, dotacion y equipos/llaves asignados al personal como activos rastreables, sustituyendo la tabla de ganchos y los cuadernos fisicos.</t>
+          <t xml:space="preserve">El nucleo es la asignacion de equipos y dotacion como activos al empleado (modelo Maintenance), que da trazabilidad a uniformes, equipos y llaves y sustituye la tabla de ganchos y los cuadernos fisicos; el flujo formal de entrega/devolucion y el control de llaves fisicas no son dedicados y requieren configuracion/desarrollo.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="2">
@@ -7197,28 +6838,12 @@
       </c>
       <c r="G43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/hr/employees/equipment] [DEV:flujo-entrega-devolucion-llaves]</t>
+          <t xml:space="preserve">Equipos/dotacion como activos asignables nativo (modelo Maintenance); flujo formal entrega/devolucion y llaves fisicas no dedicado.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] Inventario y control de uniformes; entrega de dotacion de equipos.
-[AFJ] El resguardo de llaves se lleva en una tabla fisica de ganchos sin registro de control; el resguardo de equipos asignados y la entrega de equipos danados (cuaderno fisico) carecen de trazabilidad sistematizada.</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Equipos/dotacion como activos asignables nativo (modelo Maintenance); flujo formal entrega/devolucion y llaves fisicas no dedicado.</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/hr/employees/equipment.html</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7245,7 +6870,7 @@
       </c>
       <c r="E44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Controlar la vigencia de los certificados sanitarios del personal de A&amp;B con actividades programadas que alerten antes del vencimiento.</t>
+          <t xml:space="preserve">Uso de la alerta de vencimiento nativa del maestro de empleado (actividades programadas) para controlar la vigencia de los certificados de manipulacion de alimentos y de salud del personal de A&amp;B, sustituyendo la revision mensual manual y preparando al area ante visitas de Sanidad.</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="2">
@@ -7255,27 +6880,12 @@
       </c>
       <c r="G44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/hr/employees/new_employee] [ODOO:19.0/essentials/activities]</t>
+          <t xml:space="preserve">Alerta de vencimiento nativa para permiso/visa (Expires on + Notice Period); certificados sanitarios via mismo mecanismo o Activities.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] Se controla mensualmente la vigencia de certificados de manipulacion de alimentos y de salud del personal de A&amp;B, preparando al area ante visitas de Sanidad.</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Alerta de vencimiento nativa para permiso/visa (Expires on + Notice Period); certificados sanitarios via mismo mecanismo o Activities.</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/hr/employees/new_employee.html</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7302,7 +6912,7 @@
       </c>
       <c r="E45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Gestionar el ciclo de pasantes (convenio, expediente, horarios, evaluacion final y reporte) como un flujo registrado del area de personal.</t>
+          <t xml:space="preserve">El nucleo combina los modulos nativos de reclutamiento, empleados y evaluacion para llevar el ciclo de pasantes (expediente, horarios, evaluacion final y reporte) como un flujo registrado; el convenio de pasantia especifico con universidades requiere configuracion/desarrollo.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="2">
@@ -7312,27 +6922,12 @@
       </c>
       <c r="G45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/hr/recruitment] [ODOO:19.0/hr/employees] [DEV:convenio-pasantia]</t>
+          <t xml:space="preserve">Pasantes se modela con Recruitment+Employees+Appraisals; el convenio de pasantia especifico = config/desarrollo.</t>
         </is>
       </c>
       <c r="H45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] Entrevistas con universidades y solicitud de documentacion; elaboracion de horarios semanales de pasantes; evaluacion final, carta de culminacion y reporte a la coordinacion universitaria.</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Pasantes se modela con Recruitment+Employees+Appraisals; el convenio de pasantia especifico = config/desarrollo.</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/hr/recruitment.html</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7359,7 +6954,7 @@
       </c>
       <c r="E46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Marcar el soporte a la gestion de Seguridad y Salud Laboral (politicas SST y comite ante INPSASEL); capacidad regulatoria sin via nativa identificada.</t>
+          <t xml:space="preserve">Capacidad regulatoria sin via nativa: el cumplimiento SST y el comite ante INPSASEL requieren desarrollo; los modulos de gestion documental y encuestas pueden soportar la evidencia y los registros, pero el cumplimiento en si no es cubierto por Odoo de forma estandar.</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="2">
@@ -7369,27 +6964,12 @@
       </c>
       <c r="G46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[DEV:SST-INPSASEL-VE]</t>
+          <t xml:space="preserve">Cumplimiento SST/comite INPSASEL es regulatorio VE; Documents/Surveys soportan evidencia pero el cumplimiento no es nativo.</t>
         </is>
       </c>
       <c r="H46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] La gestion de politicas SST y el comite de seguridad ante el INPSASEL estan en fase de implementacion, gestionados de forma reactiva y sin plataforma especializada.</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Cumplimiento SST/comite INPSASEL es regulatorio VE; Documents/Surveys soportan evidencia pero el cumplimiento no es nativo.</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">(regulatorio VE)</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7416,7 +6996,7 @@
       </c>
       <c r="E47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Soportar la comunicacion interna, el reporte de incidencias y las comunicaciones de cumpleanos/agasajos con mensajeria interna y actividades programadas, reduciendo la dependencia de WhatsApp como primer canal.</t>
+          <t xml:space="preserve">Uso de la mensajeria interna nativa (canales y mensajes directos) y las actividades programadas para la coordinacion interna, el reporte de novedades y las comunicaciones de cumpleanos/agasajos, dejando trazo de las novedades en el sistema y reduciendo la dependencia de WhatsApp como primer canal.</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="2">
@@ -7426,27 +7006,12 @@
       </c>
       <c r="G47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/productivity/discuss] [ODOO:19.0/essentials/activities]</t>
+          <t xml:space="preserve">Discuss (canales/DM) + Activities programadas nativo; cumpleanos via automatizacion sobre Employees.</t>
         </is>
       </c>
       <c r="H47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[RRH] La coordinacion interna y el reporte de novedades parten de WhatsApp y se formalizan por correo solo despues, con riesgo de novedades que no llegan en tiempo real.</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Discuss (canales/DM) + Activities programadas nativo; cumpleanos via automatizacion sobre Employees.</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/productivity/discuss.html</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7473,7 +7038,7 @@
       </c>
       <c r="E48" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Gestionar reservas, check-in/out, datos de huesped, disponibilidad y estado de limpieza/mantenimiento de habitaciones en un PMS hotelero sobre Odoo, sustituyendo Cloudbeds y resolviendo el estado de habitaciones no confiable.</t>
+          <t xml:space="preserve">Odoo 19 no tiene PMS hotelero oficial: la gestion de reservas, check-in/out, datos de huesped, disponibilidad y estado de limpieza/mantenimiento de habitacion requiere via OCA, modulo de tercero o desarrollo, que sustituiria a Cloudbeds y resolveria el estado de habitacion no confiable que hoy obliga a verificar fisicamente.</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="2">
@@ -7483,28 +7048,12 @@
       </c>
       <c r="G48" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[DEV:PMS-hotel-OCA-o-terceros]</t>
+          <t xml:space="preserve">Odoo 19 no tiene PMS hotelero oficial; via OCA (pms) o terceros o desarrollo.</t>
         </is>
       </c>
       <c r="H48" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[GHO] Ama de Llaves no actualiza Cloudbeds en tiempo real, por lo que recepcion debe verificar fisicamente; se reporto la venta de una habitacion sin colchon retirado para mantenimiento.
-[GHO] El registro de huespedes esta descrito paso a paso para entrada por puerta y con reserva previa, con captura de datos de identidad, adjuntos y firma de normativas.</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Odoo 19 no tiene PMS hotelero oficial; via OCA (pms) o terceros o desarrollo.</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">(sin app hotel oficial)</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7531,7 +7080,7 @@
       </c>
       <c r="E49" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Vender en las tiendas con un punto de venta enlazado a inventario que descuente stock y disponga de un perfil de cliente generico para visitantes, eliminando la venta en papel y el descuadre de inventario.</t>
+          <t xml:space="preserve">Punto de venta de tienda cuyo nucleo enlazado a inventario es nativo (descuento automatico de stock y cliente generico para visitantes) y que elimina la venta en papel ajustada a mano en Cloudbeds y el descuadre de inventario; la emision del documento fiscal venezolano requiere desarrollo/integracion de localizacion fiscal sobre ese nucleo.</t>
         </is>
       </c>
       <c r="F49" t="inlineStr" s="2">
@@ -7541,28 +7090,12 @@
       </c>
       <c r="G49" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[DEV:pos-tienda-fiscal-ve]</t>
+          <t xml:space="preserve">POS de tienda enlazado a inventario es nativo, pero la VENTA emite documento fiscal: El nucleo POS de Odoo es nativo, pero la emision fiscal venezolana (maquina/impresora fiscal homologada, IGTF en ticket, correlativos y formatos fiscales) NO es nativa; requiere desarrollo/integracion de localizacion fiscal VE.</t>
         </is>
       </c>
       <c r="H49" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[GHO] Las ventas de tienda a visitantes externos se anotan en papel y se ajustan manualmente en Cloudbeds porque no existe un perfil de cliente visitante, lo que descuadra el inventario.
-[GHO] Mercancia comprada por el dueno entra a las tiendas sin factura ni paso por almacen, y la Tienda Playera cobra a cuenta externa del propietario con recibo en papel.</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">POS de tienda enlazado a inventario es nativo, pero la VENTA emite documento fiscal: El nucleo POS de Odoo es nativo, pero la emision fiscal venezolana (maquina/impresora fiscal homologada, IGTF en ticket, correlativos y formatos fiscales) NO es nativa; requiere desarrollo/integracion de localizacion fiscal VE.</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/sales/point_of_sale/use.html (nucleo no-fiscal)</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7589,7 +7122,7 @@
       </c>
       <c r="E50" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Marcar la integracion de la programacion de llaves electronicas de habitacion (TT Hotel/Time Locks); capacidad de hardware externo sin via nativa Odoo.</t>
+          <t xml:space="preserve">Capacidad de hardware externo sin via nativa: la programacion de llaves electronicas de habitacion (TT Hotel/Time Locks/Lockia) requiere desarrollo de integracion a medida con las cerraduras, no cubierto por Odoo de forma estandar.</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="2">
@@ -7599,27 +7132,12 @@
       </c>
       <c r="G50" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[DEV:integracion-cerraduras-TTHotel]</t>
+          <t xml:space="preserve">Programacion de llaves electronicas (TT Hotel): integracion de hardware a medida.</t>
         </is>
       </c>
       <c r="H50" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[GHO] Las llaves se programan en TT Hotel o en Time Locks/Lockia segun el tipo de cerradura de la habitacion, con la operacion en transicion hacia cerraduras inteligentes.</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Programacion de llaves electronicas (TT Hotel): integracion de hardware a medida.</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">(hardware externo)</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7646,7 +7164,7 @@
       </c>
       <c r="E51" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Centralizar los canales de atencion (mensajeria, correo, telefono) y la gestion de prospectos en un flujo unico con conversion a reserva, conservando la asistencia automatizada y el modo manual de respaldo.</t>
+          <t xml:space="preserve">El nucleo son los modulos nativos de CRM y chat en vivo que centralizan mensajeria, correo y telefono y convierten la conversacion en prospecto en un pipeline unico, conservando la asistencia automatizada y el modo manual de respaldo; la conversion del prospecto a reserva depende del PMS, por lo que esa parte no es nativa y requiere desarrollo.</t>
         </is>
       </c>
       <c r="F51" t="inlineStr" s="2">
@@ -7656,28 +7174,12 @@
       </c>
       <c r="G51" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/sales/crm] [ODOO:19.0/websites/livechat] [DEV:conversion-a-reserva]</t>
+          <t xml:space="preserve">CRM (pipeline) + Live Chat (comando /lead) nativo; conversion a reserva depende de PMS (no nativo).</t>
         </is>
       </c>
       <c r="H51" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[GHO] Visito unifica WhatsApp e Instagram con respuesta por IA y modo manual de respaldo, con conversion a reserva en Cloudbeds.
-[GHO] La IA de Visito responde solicitudes operativas de huespedes hospedados sin que recepcion las vea a tiempo, y no hay telefono en habitacion.</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">CRM (pipeline) + Live Chat (comando /lead) nativo; conversion a reserva depende de PMS (no nativo).</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/sales/crm.html</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7704,7 +7206,7 @@
       </c>
       <c r="E52" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Complementar la resolucion reactiva de quejas con un instrumento de medicion de satisfaccion del huesped.</t>
+          <t xml:space="preserve">Uso del modulo de encuestas nativo (envio, scoring y analisis) como instrumento documentado de medicion de satisfaccion del huesped, que sustituye la gestion puramente reactiva de quejas por un dato estructurado y consultable.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr" s="2">
@@ -7714,27 +7216,12 @@
       </c>
       <c r="G52" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/marketing/surveys]</t>
+          <t xml:space="preserve">Encuestas de satisfaccion con envio, scoring y analisis, nativo.</t>
         </is>
       </c>
       <c r="H52" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[GHO] La satisfaccion del cliente se gestiona reactivamente, sin instrumento documentado de medicion.</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Encuestas de satisfaccion con envio, scoring y analisis, nativo.</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/marketing/surveys.html</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7761,7 +7248,7 @@
       </c>
       <c r="E53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Soportar la capacitacion del personal nuevo sobre los sistemas y normativas con material disponible y vigente, reduciendo la dependencia de la memoria de un solo rol.</t>
+          <t xml:space="preserve">Uso del modulo de formacion nativo (cursos con contenidos, evaluaciones y certificacion) para la capacitacion del personal nuevo sobre sistemas y normativas, que centraliza un instructivo vigente y disponible y reduce la dependencia de la memoria y disponibilidad de un solo rol.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr" s="2">
@@ -7771,27 +7258,12 @@
       </c>
       <c r="G53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/websites/elearning]</t>
+          <t xml:space="preserve">Cursos con contenidos, quiz y certificacion, nativo.</t>
         </is>
       </c>
       <c r="H53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[GHO] No existe instructivo actualizado y disponible; la orientacion depende de la memoria y disponibilidad del rol gerencial.</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Cursos con contenidos, quiz y certificacion, nativo.</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/websites/elearning.html</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7818,7 +7290,7 @@
       </c>
       <c r="E54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Capturar las solicitudes de reparacion como ordenes de mantenimiento con estado y responsable, dando trazabilidad al tiempo de respuesta y al cierre, incluyendo reparaciones con tecnico externo.</t>
+          <t xml:space="preserve">Uso del modulo de mantenimiento nativo para capturar las solicitudes de reparacion como ordenes con responsable y etapas, que centraliza en el sistema lo que hoy llega por WhatsApp, radio o de forma verbal y da trazabilidad del tiempo de respuesta y del cierre, incluyendo las reparaciones con tecnico externo.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr" s="2">
@@ -7828,28 +7300,12 @@
       </c>
       <c r="G54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/maintenance/maintenance_requests]</t>
+          <t xml:space="preserve">Solicitudes de mantenimiento con responsable y etapas, trazabilidad de cierre nativo.</t>
         </is>
       </c>
       <c r="H54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[OPE] Las solicitudes de gerencia y de los demas departamentos se reciben por WhatsApp, radio o de forma verbal y no se cargan a ninguna plataforma; no hay trazabilidad del tiempo de respuesta ni del cierre de la falla.
-[GHO] Cada reparacion con tecnico externo se gestiona ad hoc; el tecnico a veces actua de forma autonoma sin notificar, y no hay registro que de seguimiento desde la deteccion del dano hasta el pago.</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Solicitudes de mantenimiento con responsable y etapas, trazabilidad de cierre nativo.</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/inventory_and_mrp/maintenance/maintenance_requests.html</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7876,7 +7332,7 @@
       </c>
       <c r="E55" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Registrar los equipos criticos como activos con planes de mantenimiento preventivo por tiempo o uso, sustituyendo la dependencia del criterio individual y la verificacion manual.</t>
+          <t xml:space="preserve">El nucleo es el modulo de mantenimiento nativo que registra los equipos criticos como activos con planes preventivos por tiempo (MTBF), sustituyendo el trabajo reactivo basado en el criterio del operador; el preventivo por uso/medidor no esta documentado como nativo y requiere configuracion/desarrollo.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr" s="2">
@@ -7886,27 +7342,12 @@
       </c>
       <c r="G55" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/maintenance/add_new_equipment] [DEV:preventivo-por-uso-medidor]</t>
+          <t xml:space="preserve">Equipos + preventivo por tiempo (MTBF) nativo; preventivo por uso/medidor no documentado nativo.</t>
         </is>
       </c>
       <c r="H55" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[OPE] La planificacion electrica y la atencion de fallas son mayormente reactivas; el trabajo preventivo depende del criterio del operador y no de un calendario por tiempo de uso de los activos.</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Equipos + preventivo por tiempo (MTBF) nativo; preventivo por uso/medidor no documentado nativo.</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/inventory_and_mrp/maintenance/add_new_equipment.html</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7933,7 +7374,7 @@
       </c>
       <c r="E56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Gestionar la solicitud y recepcion de los servicios basicos (agua, gasoil, gas) como orden de compra y recepcion de inventario con control de niveles, sustituyendo la lectura manual y la solicitud bajo demanda.</t>
+          <t xml:space="preserve">Uso de la orden de compra y la recepcion de inventario nativas para gestionar agua, gasoil y gas con control de niveles de stock, que anticipa la reposicion y sustituye la lectura manual y la solicitud bajo demanda que hoy expone al hotel a quedarse sin autonomia energetica o sin gas.</t>
         </is>
       </c>
       <c r="F56" t="inlineStr" s="2">
@@ -7943,25 +7384,10 @@
       </c>
       <c r="G56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/purchase/purchase-order] [ODOO:19.0/inventory/delivery-picking]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H56" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[OPE] La gestion de niveles de gasoil/gas por lectura manual y solicitud bajo demanda expone al hotel a quedarse sin autonomia energetica o sin gas para cocinas si el proveedor se retrasa.</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7990,7 +7416,7 @@
       </c>
       <c r="E57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Generar el reporte regulatorio diario de ocupacion e ingresos para Venetur e INATUR a partir de los datos del sistema, reduciendo la reconstruccion nocturna y manual que cruza dos sistemas.</t>
+          <t xml:space="preserve">No existe reporte Venetur/INATUR nativo: aunque los ingresos por categoria salen de contabilidad y POS, los indicadores de ocupacion dependen del PMS, por lo que generar el reporte regulatorio diario requiere desarrollo que consolide ambas fuentes y elimine la reconstruccion nocturna y manual en el formato Excel del organismo.</t>
         </is>
       </c>
       <c r="F57" t="inlineStr" s="2">
@@ -8000,28 +7426,12 @@
       </c>
       <c r="G57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[DEV:reporte-venetur-inatur]</t>
+          <t xml:space="preserve">No existe reporte Venetur/INATUR nativo; ingresos salen de Accounting/POS pero ocupacion requiere PMS.</t>
         </is>
       </c>
       <c r="H57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[AFL] El reporte diario a Venetur consolida a mano, en el formato Excel del organismo, los ingresos por categoria de Odoo y los indicadores de ocupacion de Cloudbeds, con plazos nocturnos estrictos en temporada alta.
-[CCS] El cruce de pagos, EDR e informe de obras a Venetur se prepara manualmente, lo que el equipo identifica como riesgo de actas de reparo en futuras revisiones.</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">No existe reporte Venetur/INATUR nativo; ingresos salen de Accounting/POS pero ocupacion requiere PMS.</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">(reporte regulatorio VE)</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -8048,7 +7458,7 @@
       </c>
       <c r="E58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Marcar la administracion de cuentas y usuarios de las plataformas bancarias con un responsable unico y niveles de aprobacion, separada de la operacion que controla; gestion de acceso externo sin via nativa.</t>
+          <t xml:space="preserve">Gestion de acceso externo sin via nativa: la administracion de cuentas y usuarios de las plataformas bancarias vive fuera de Odoo, por lo que se aborda como definicion de un responsable unico y niveles de aprobacion separados de la operacion que controla, no como capacidad del sistema.</t>
         </is>
       </c>
       <c r="F58" t="inlineStr" s="2">
@@ -8058,28 +7468,12 @@
       </c>
       <c r="G58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[DEV:gestion-usuarios-banca]</t>
+          <t xml:space="preserve">Administracion de cuentas/usuarios de plataformas bancarias es externo a Odoo.</t>
         </is>
       </c>
       <c r="H58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[CTR] La gestion del usuario master esta dividida entre dos roles (Contraloria y Administracion y Finanzas) sin responsable unico ni niveles de aprobacion definidos.
-[CCS] Apertura de cuentas juridicas y de cuentas nominas.</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Administracion de cuentas/usuarios de plataformas bancarias es externo a Odoo.</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">(externo banca)</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -8106,7 +7500,7 @@
       </c>
       <c r="E59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conciliar las ventas y cuotas gestionadas por Cashea y los lotes de Credicard contra los recibos de cobro y la posicion financiera, formalizando el seguimiento del cierre de lote de los puntos de venta.</t>
+          <t xml:space="preserve">Uso de la facturacion y los recibos de cobro nativos para conciliar las ventas y cuotas de Cashea y los lotes de Credicard contra la posicion financiera, formalizando en el sistema el seguimiento del cierre de lote de cada punto de venta y el cobro por morosidad.</t>
         </is>
       </c>
       <c r="F59" t="inlineStr" s="2">
@@ -8116,26 +7510,10 @@
       </c>
       <c r="G59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/accounting/customer-invoice]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H59" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[CCS] Verificacion de ordenes y seguimiento de cuotas de ventas del hotel; posicion financiera 4% a pagar / cobro por morosidad.
-[CCS] Seguimiento y actualizacion de puntos de venta del hotel; cierre de lote de puntos de venta.</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8164,7 +7542,7 @@
       </c>
       <c r="E60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Facturar entre las companias del grupo (Eracon Salud/Alimentos y SERAC) con la facturacion entre companias, sustituyendo la actualizacion manual del inventario intercompany.</t>
+          <t xml:space="preserve">Uso de la facturacion entre companias nativa para las operaciones recurrentes entre Eracon Alimentos/Salud y SERAC, que genera de forma cruzada la factura y el movimiento en la otra compania y sustituye la actualizacion manual del inventario intercompany.</t>
         </is>
       </c>
       <c r="F60" t="inlineStr" s="2">
@@ -8174,25 +7552,10 @@
       </c>
       <c r="G60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/accounting/customer-invoice]</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H60" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[CCS] La facturacion recurrente de Eracon Alimentos a SERAC y la eventual de Eracon Salud corresponde a la facturacion entre companias de Odoo.</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8221,7 +7584,7 @@
       </c>
       <c r="E61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Soportar la supervision de control de gestion con cuestionarios periodicos por departamento, plan de trabajo y seguimiento de hallazgos y novedades, sustituyendo Word, WhatsApp y el escalamiento informal.</t>
+          <t xml:space="preserve">Uso de los modulos nativos de encuestas y de proyectos para la supervision de control de gestion (cuestionarios periodicos por departamento, plan de trabajo y seguimiento de hallazgos al cierre), que consolida los resultados en tiempo real y sustituye el registro en Word, la comunicacion por WhatsApp y el escalamiento informal.</t>
         </is>
       </c>
       <c r="F61" t="inlineStr" s="2">
@@ -8231,28 +7594,12 @@
       </c>
       <c r="G61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[ODOO:19.0/marketing/surveys] [ODOO:19.0/services/project]</t>
+          <t xml:space="preserve">Cuestionarios periodicos (Surveys) + plan de trabajo/seguimiento (Project) nativo.</t>
         </is>
       </c>
       <c r="H61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[CTR] La validacion de gestion por departamento se registra en Word y se comunica por llamada o WhatsApp, sin consolidacion ni resultados en tiempo real.
-[AFJ] El analista detecta, reporta, asigna actividad en Odoo y da seguimiento al cierre de errores de pedidos/facturas originados por otros departamentos.</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Cuestionarios periodicos (Surveys) + plan de trabajo/seguimiento (Project) nativo.</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">https://www.odoo.com/documentation/19.0/applications/marketing/surveys.html</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -8279,7 +7626,7 @@
       </c>
       <c r="E62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Marcar la administracion de usuarios, clientes y metodos de pago de los sistemas de punto de servicio (Cloudbeds, Poster) en tanto persistan como sistemas externos; configuracion de terceros sin via nativa Odoo.</t>
+          <t xml:space="preserve">Configuracion de terceros sin via nativa: mientras persistan Cloudbeds y Poster como sistemas externos, la administracion de sus usuarios, clientes y metodos de pago se mantiene fuera de Odoo y solo una integracion a medida la acercaria al sistema; de migrar a POS/PMS sobre Odoo se absorberia en sus maestros.</t>
         </is>
       </c>
       <c r="F62" t="inlineStr" s="2">
@@ -8289,27 +7636,12 @@
       </c>
       <c r="G62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[DEV:integracion-Cloudbeds-Poster]</t>
+          <t xml:space="preserve">Administracion de Cloudbeds/Poster: sistemas externos, integracion a medida mientras persistan.</t>
         </is>
       </c>
       <c r="H62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[AFL] Creacion de usuarios en Cloudbeds; configuracion de metodos de pago en Cloudbeds; creacion de usuarios y clientes en Poster.</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Administracion de Cloudbeds/Poster: sistemas externos, integracion a medida mientras persistan.</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">(sistemas externos)</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -8336,7 +7668,7 @@
       </c>
       <c r="E63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Marcar como fuera del alcance de Odoo las tareas operativas puramente fisicas y el soporte ofimatico general (limpieza, montaje, jardineria, piscina, copias, atencion general); no requieren capacidad del sistema y se documentan para descarte.</t>
+          <t xml:space="preserve">Fuera del alcance de Odoo: las tareas operativas puramente fisicas y el soporte ofimatico general (limpieza, montaje, jardineria, piscina, copias, atencion general) no implican transaccion ni dato maestro y no son objeto del sistema; se documentan para descarte explicito.</t>
         </is>
       </c>
       <c r="F63" t="inlineStr" s="2">
@@ -8346,29 +7678,12 @@
       </c>
       <c r="G63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[FUERA-DE-ALCANCE]</t>
+          <t xml:space="preserve">Tareas fisicas (limpieza, jardineria, piscina) y ofimatica general: no son objeto de Odoo.</t>
         </is>
       </c>
       <c r="H63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">[OPE] Las rutinas diarias de mantenimiento (medicion de cloro/pH, aspiracion y retrolavado, activacion de bombas, limpieza de areas verdes y recoleccion de residuos) tienen disparador, frecuencia y pasos definidos.
-[AFJ] Operaciones de soporte administrativo (copias, sello, POS, equipos) y atencion y asesoramiento al personal y terceros en procesos.
-[BAR] Todas las fases se cierran con limpieza del area y una entrega de guardia que comunica pendientes al turno entrante.</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Tareas fisicas (limpieza, jardineria, piscina) y ofimatica general: no son objeto de Odoo.</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">(n/a)</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>

</xml_diff>